<commit_message>
Add monthly package schedule and tax treatment
</commit_message>
<xml_diff>
--- a/projects/PetroUrdaneta-FDP9/compensation/modelo_paquetes_personal_2_etapas.xlsx
+++ b/projects/PetroUrdaneta-FDP9/compensation/modelo_paquetes_personal_2_etapas.xlsx
@@ -11,15 +11,18 @@
     <sheet name="Resumen" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Supuestos" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Personal" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Definiciones" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Mensual" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Definiciones" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Definiciones!$B$2:$K$34</definedName>
+    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">Definiciones!$B$2:$K$34</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Mensual!$B$2:$T$29</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Titles" vbProcedure="false">Mensual!$10:$10</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">Personal!$B$2:$AF$21</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">Personal!$10:$10</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Personal!$C$10:$AF$19</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Resumen!$B$2:$R$45</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Supuestos!$B$2:$J$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Supuestos!$B$2:$J$38</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -135,7 +138,73 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D16" authorId="0">
+    <comment ref="D12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Fuente: supuesto presupuestario del modelo preparado el 5 de septiembre de 2026. Supuesto gerencial: el repatriado asume su impuesto personal. Ajustar si existen contribuciones patronales obligatorias u otras cargas de la empresa.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>8</xdr:row>
+                <xdr:rowOff>10</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Fuente: supuesto presupuestario del modelo preparado el 5 de septiembre de 2026. Supuesto gerencial: la empresa cubre o neutraliza el impuesto del país de trabajo para el expatriado. No incluye obligaciones del país de origen salvo política expresa.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D18" authorId="0">
       <text>
         <r>
           <rPr>
@@ -168,7 +237,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D17" authorId="0">
+    <comment ref="D19" authorId="0">
       <text>
         <r>
           <rPr>
@@ -201,7 +270,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D18" authorId="0">
+    <comment ref="D20" authorId="0">
       <text>
         <r>
           <rPr>
@@ -226,15 +295,15 @@
                 <xdr:col>1</xdr:col>
                 <xdr:colOff>55</xdr:colOff>
                 <xdr:row>8</xdr:row>
-                <xdr:rowOff>3</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="D19" authorId="0">
+                <xdr:rowOff>4</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D21" authorId="0">
       <text>
         <r>
           <rPr>
@@ -4440,7 +4509,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="215">
   <si>
     <t xml:space="preserve">Resumen ejecutivo — Paquetes de personal</t>
   </si>
@@ -4553,13 +4622,13 @@
     <t xml:space="preserve">Selección actual por persona</t>
   </si>
   <si>
-    <t xml:space="preserve">Todos expatriados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Todos repatriados — con housing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Todos repatriados — sin housing</t>
+    <t xml:space="preserve">Todos expatriados — empresa cubre impuesto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todos repatriados — con housing; empleado paga impuesto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todos repatriados — sin housing; empleado paga impuesto</t>
   </si>
   <si>
     <t xml:space="preserve">DETALLE EJECUTIVO POR PERSONA</t>
@@ -4598,10 +4667,10 @@
     <t xml:space="preserve">3. Validar la política inicial: Caracas con housing; Maracaibo sin housing para repatriados.</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Incorporar costos únicos cotizados: viaje, mudanza, permisos, asesoría, alojamiento temporal y settling-in.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Obtener dictamen escrito de inmigración, laboral y fiscal antes de implementar la etapa de consultoría.</t>
+    <t xml:space="preserve">4. Confirmar por escrito que el expatriado recibe protección / gross-up fiscal y que el repatriado asume su impuesto personal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Incorporar costos únicos cotizados y obtener dictamen escrito de inmigración, laboral y fiscal.</t>
   </si>
   <si>
     <t xml:space="preserve">Supuestos y política de paquetes</t>
@@ -4625,6 +4694,12 @@
     <t xml:space="preserve">Factor de Tax &amp; Social en la etapa 1</t>
   </si>
   <si>
+    <t xml:space="preserve">Factor de Tax &amp; Social pagado por la empresa — Repatriado M7+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factor de Tax &amp; Social pagado por la empresa — Expatriado M7+</t>
+  </si>
+  <si>
     <t xml:space="preserve">POLÍTICA AUTOMÁTICA DE VIVIENDA POR CIUDAD</t>
   </si>
   <si>
@@ -4733,10 +4808,22 @@
     <t xml:space="preserve">Vehículo</t>
   </si>
   <si>
-    <t xml:space="preserve">Tax &amp; Social</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M1–M6 usa factor 0%; M7+ conserva el valor anual prorrateado.</t>
+    <t xml:space="preserve">Impuesto del país de trabajo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No cubierto en el modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lo asume el empleado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lo cubre / neutraliza la empresa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factores editables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repatriado: factor empresa 0%; expatriado: factor empresa 100% por defecto.</t>
   </si>
   <si>
     <t xml:space="preserve">Costos únicos de transición</t>
@@ -4945,6 +5032,81 @@
     <t xml:space="preserve">TOTAL — 9 POSICIONES</t>
   </si>
   <si>
+    <t xml:space="preserve">Costo mensual por persona</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1–M6 como consultor | M7–M12 según paquete seleccionado; los costos únicos se cargan en M7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USD | Expatriado: empresa cubre / neutraliza impuesto del país de trabajo; Repatriado: empleado asume su impuesto personal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DETALLE MENSUAL POR PERSONA — ESCENARIO SELECCIONADO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tratamiento fiscal M7+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COSTO TOTAL POR MES — COMPARACIÓN DE ESCENARIOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tratamiento fiscal desde M7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Según selección individual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todos expatriados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Empresa cubre / neutraliza impuesto del país de trabajo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todos repatriados — con housing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Empleado asume impuesto personal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todos repatriados — sin housing</t>
+  </si>
+  <si>
     <t xml:space="preserve">Definición de los paquetes</t>
   </si>
   <si>
@@ -4972,7 +5134,10 @@
     <t xml:space="preserve">PAQUETE REPATRIADO — DESDE EL MES 7</t>
   </si>
   <si>
-    <t xml:space="preserve">• Compensación recurrente: salario base, seguro médico, vehículo y Tax &amp; Social.</t>
+    <t xml:space="preserve">• Compensación recurrente pagada por la empresa: salario base, seguro médico y vehículo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Impuesto personal: lo asume el repatriado. El factor de Tax &amp; Social pagado por la empresa es 0% por defecto, salvo cargas patronales obligatorias.</t>
   </si>
   <si>
     <t xml:space="preserve">• Housing: condicional. Política inicial editable: Caracas = Sí; Maracaibo = No. Un override individual prevalece sobre la regla automática.</t>
@@ -4990,7 +5155,10 @@
     <t xml:space="preserve">PAQUETE EXPATRIADO — DESDE EL MES 7</t>
   </si>
   <si>
-    <t xml:space="preserve">• Compensación recurrente: paquete anual fuente completo prorrateado — salario base, housing, seguro médico, home leave, vehículo y Tax &amp; Social.</t>
+    <t xml:space="preserve">• Compensación recurrente: salario base, housing, seguro médico, home leave y vehículo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Protección fiscal: la empresa cubre o neutraliza el impuesto del país de trabajo mediante pago, gross-up o tax equalization; el factor presupuestario es 100% del Tax &amp; Social fuente.</t>
   </si>
   <si>
     <t xml:space="preserve">• Costos únicos: incorporar, cuando correspondan, regularización migratoria, asesoría fiscal, alojamiento temporal y otros costos de movilidad no incluidos en la tabla fuente.</t>
@@ -5271,7 +5439,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="63">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5412,6 +5580,10 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="169" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5505,6 +5677,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5748,13 +5932,13 @@
                   <c:v>Selección actual por persona</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Todos expatriados</c:v>
+                  <c:v>Todos expatriados — empresa cubre impuesto</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Todos repatriados — con housing</c:v>
+                  <c:v>Todos repatriados — con housing; empleado paga impuesto</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Todos repatriados — sin housing</c:v>
+                  <c:v>Todos repatriados — sin housing; empleado paga impuesto</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5772,10 +5956,10 @@
                   <c:v>2243600</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2191600</c:v>
+                  <c:v>2038400</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2092600</c:v>
+                  <c:v>1939400</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5783,11 +5967,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="29746751"/>
-        <c:axId val="19831421"/>
+        <c:axId val="65066025"/>
+        <c:axId val="48480607"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="29746751"/>
+        <c:axId val="65066025"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5853,7 +6037,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19831421"/>
+        <c:crossAx val="48480607"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5861,7 +6045,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="19831421"/>
+        <c:axId val="48480607"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5937,7 +6121,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29746751"/>
+        <c:crossAx val="65066025"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6437,7 +6621,7 @@
         <v>1045200</v>
       </c>
       <c r="E22" s="20" t="n">
-        <f aca="false">Personal!M21/12*Supuestos!$D$10</f>
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!I11:I19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$13)/12*Supuestos!$D$10</f>
         <v>1198400</v>
       </c>
       <c r="F22" s="21" t="n">
@@ -6449,7 +6633,7 @@
         <v>153200</v>
       </c>
       <c r="H22" s="20" t="n">
-        <f aca="false">Personal!M21</f>
+        <f aca="false">E22/Supuestos!$D$10*12</f>
         <v>2396800</v>
       </c>
     </row>
@@ -6462,20 +6646,20 @@
         <v>1045200</v>
       </c>
       <c r="E23" s="20" t="n">
-        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19))/12*Supuestos!$D$10</f>
-        <v>1146400</v>
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12*Supuestos!$D$10</f>
+        <v>993200</v>
       </c>
       <c r="F23" s="21" t="n">
         <f aca="false">D23+E23</f>
-        <v>2191600</v>
+        <v>2038400</v>
       </c>
       <c r="G23" s="20" t="n">
         <f aca="false">Personal!M21-F23</f>
-        <v>205200</v>
+        <v>358400</v>
       </c>
       <c r="H23" s="20" t="n">
         <f aca="false">E23/Supuestos!$D$10*12</f>
-        <v>2292800</v>
+        <v>1986400</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6487,20 +6671,20 @@
         <v>1045200</v>
       </c>
       <c r="E24" s="24" t="n">
-        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19))/12*Supuestos!$D$10</f>
-        <v>1047400</v>
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12*Supuestos!$D$10</f>
+        <v>894200</v>
       </c>
       <c r="F24" s="25" t="n">
         <f aca="false">D24+E24</f>
-        <v>2092600</v>
+        <v>1939400</v>
       </c>
       <c r="G24" s="24" t="n">
         <f aca="false">Personal!M21-F24</f>
-        <v>304200</v>
+        <v>457400</v>
       </c>
       <c r="H24" s="24" t="n">
         <f aca="false">E24/Supuestos!$D$10*12</f>
-        <v>2094800</v>
+        <v>1788400</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6920,14 +7104,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="C3:J36"/>
+  <dimension ref="C3:J38"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="12"/>
@@ -6980,313 +7163,329 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="9" t="s">
         <v>60</v>
       </c>
       <c r="D11" s="35" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C14" s="4" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C12" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-    </row>
-    <row r="15" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C15" s="5" t="s">
+      <c r="D12" s="35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C13" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D13" s="36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C16" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C17" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C16" s="36" t="s">
+      <c r="E17" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="37" t="s">
+      <c r="F17" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E16" s="36" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="F16" s="36" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C17" s="38" t="s">
+      <c r="D18" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="D17" s="39" t="s">
+      <c r="E18" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="E17" s="38" t="s">
+      <c r="F18" s="37" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C19" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="F17" s="38" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="38" t="s">
+      <c r="D19" s="40" t="s">
         <v>72</v>
       </c>
-      <c r="D18" s="39" t="s">
-        <v>67</v>
-      </c>
-      <c r="E18" s="38" t="s">
+      <c r="E19" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="F18" s="38" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C19" s="40" t="s">
+      <c r="F19" s="39" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C20" s="39" t="s">
         <v>74</v>
       </c>
-      <c r="D19" s="41" t="s">
-        <v>74</v>
-      </c>
-      <c r="E19" s="40" t="s">
+      <c r="D20" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="E20" s="39" t="s">
         <v>75</v>
       </c>
-      <c r="F19" s="40" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C22" s="4" t="s">
+      <c r="F20" s="39" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C21" s="41" t="s">
         <v>76</v>
       </c>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-    </row>
-    <row r="23" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C23" s="5" t="s">
+      <c r="D21" s="42" t="s">
+        <v>76</v>
+      </c>
+      <c r="E21" s="41" t="s">
         <v>77</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="F21" s="41" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C24" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C25" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="D25" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="G23" s="5" t="s">
+      <c r="E25" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H23" s="5" t="s">
+      <c r="F25" s="5" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C24" s="8" t="s">
+      <c r="G25" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="H25" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E24" s="8" t="s">
+    </row>
+    <row r="26" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C26" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="D26" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="G24" s="8" t="s">
+      <c r="E26" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="H24" s="8" t="s">
+      <c r="F26" s="8" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C25" s="11" t="s">
+      <c r="G26" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D25" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="E25" s="11" t="s">
+      <c r="H26" s="8" t="s">
         <v>90</v>
-      </c>
-      <c r="F25" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="G25" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="H25" s="11" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C26" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="E26" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="F26" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="G26" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="H26" s="11" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C27" s="11" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C28" s="11" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C29" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="E29" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="F29" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="H29" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="D29" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="E29" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="F29" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="G29" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="H29" s="11" t="s">
+    </row>
+    <row r="30" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C30" s="11" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="30" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C30" s="16" t="s">
+      <c r="D30" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="E30" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="H30" s="11" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C31" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="D30" s="16" t="s">
+      <c r="D31" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="E30" s="16" t="s">
+      <c r="E31" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="F30" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="G30" s="16" t="s">
+      <c r="F31" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="H30" s="16" t="s">
+      <c r="G31" s="11" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C33" s="4" t="s">
+      <c r="H31" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-    </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C34" s="42" t="s">
+    </row>
+    <row r="32" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C32" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="D34" s="42"/>
-      <c r="E34" s="42"/>
-      <c r="F34" s="42"/>
-      <c r="G34" s="42"/>
-      <c r="H34" s="42"/>
-      <c r="I34" s="42"/>
-      <c r="J34" s="42"/>
-    </row>
-    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C35" s="42"/>
-      <c r="D35" s="42"/>
-      <c r="E35" s="42"/>
-      <c r="F35" s="42"/>
-      <c r="G35" s="42"/>
-      <c r="H35" s="42"/>
-      <c r="I35" s="42"/>
-      <c r="J35" s="42"/>
+      <c r="D32" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="E32" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="F32" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="G32" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="H32" s="16" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C35" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
+      <c r="I35" s="4"/>
+      <c r="J35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C36" s="42"/>
-      <c r="D36" s="42"/>
-      <c r="E36" s="42"/>
-      <c r="F36" s="42"/>
-      <c r="G36" s="42"/>
-      <c r="H36" s="42"/>
-      <c r="I36" s="42"/>
-      <c r="J36" s="42"/>
+      <c r="C36" s="43" t="s">
+        <v>111</v>
+      </c>
+      <c r="D36" s="43"/>
+      <c r="E36" s="43"/>
+      <c r="F36" s="43"/>
+      <c r="G36" s="43"/>
+      <c r="H36" s="43"/>
+      <c r="I36" s="43"/>
+      <c r="J36" s="43"/>
+    </row>
+    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C37" s="43"/>
+      <c r="D37" s="43"/>
+      <c r="E37" s="43"/>
+      <c r="F37" s="43"/>
+      <c r="G37" s="43"/>
+      <c r="H37" s="43"/>
+      <c r="I37" s="43"/>
+      <c r="J37" s="43"/>
+    </row>
+    <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C38" s="43"/>
+      <c r="D38" s="43"/>
+      <c r="E38" s="43"/>
+      <c r="F38" s="43"/>
+      <c r="G38" s="43"/>
+      <c r="H38" s="43"/>
+      <c r="I38" s="43"/>
+      <c r="J38" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="C3:J3"/>
     <mergeCell ref="C8:F8"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C33:J33"/>
-    <mergeCell ref="C34:J36"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C35:J35"/>
+    <mergeCell ref="C36:J38"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.5"/>
@@ -7338,7 +7537,7 @@
   <sheetData>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="1" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -7372,17 +7571,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C6" s="3" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C8" s="4" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -7416,7 +7615,7 @@
     </row>
     <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C10" s="5" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>42</v>
@@ -7425,1158 +7624,1158 @@
         <v>41</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="P10" s="5" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="R10" s="5" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="S10" s="5" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="T10" s="5" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="U10" s="5" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="V10" s="5" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="X10" s="5" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="Y10" s="5" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="Z10" s="5" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="AA10" s="5" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="AB10" s="5" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="AC10" s="5" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="AD10" s="5" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="AE10" s="5" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="AF10" s="5" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C11" s="43" t="n">
+      <c r="C11" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="44" t="s">
-        <v>138</v>
-      </c>
-      <c r="E11" s="44" t="s">
-        <v>139</v>
-      </c>
-      <c r="F11" s="45" t="n">
+      <c r="D11" s="45" t="s">
+        <v>144</v>
+      </c>
+      <c r="E11" s="45" t="s">
+        <v>145</v>
+      </c>
+      <c r="F11" s="46" t="n">
         <v>360000</v>
       </c>
-      <c r="G11" s="46" t="n">
+      <c r="G11" s="47" t="n">
         <v>36000</v>
       </c>
-      <c r="H11" s="46" t="n">
+      <c r="H11" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="I11" s="46" t="n">
+      <c r="I11" s="47" t="n">
         <v>20000</v>
       </c>
-      <c r="J11" s="46" t="n">
+      <c r="J11" s="47" t="n">
         <v>24000</v>
       </c>
-      <c r="K11" s="46" t="n">
+      <c r="K11" s="47" t="n">
         <v>72000</v>
       </c>
-      <c r="L11" s="47" t="n">
+      <c r="L11" s="48" t="n">
         <f aca="false">SUM(F11:K11)</f>
         <v>524000</v>
       </c>
-      <c r="M11" s="46" t="n">
+      <c r="M11" s="47" t="n">
         <v>524000</v>
       </c>
-      <c r="N11" s="48" t="n">
+      <c r="N11" s="49" t="n">
         <f aca="false">L11-M11</f>
         <v>0</v>
       </c>
-      <c r="O11" s="49" t="n">
+      <c r="O11" s="50" t="n">
         <f aca="false">F11/12*Supuestos!$D$9</f>
         <v>180000</v>
       </c>
-      <c r="P11" s="50" t="n">
+      <c r="P11" s="51" t="n">
         <f aca="false">G11/12*Supuestos!$D$9</f>
         <v>18000</v>
       </c>
-      <c r="Q11" s="50" t="n">
+      <c r="Q11" s="51" t="n">
         <f aca="false">H11/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="R11" s="50" t="n">
+      <c r="R11" s="51" t="n">
         <f aca="false">I11/12*Supuestos!$D$9</f>
         <v>10000</v>
       </c>
-      <c r="S11" s="50" t="n">
+      <c r="S11" s="51" t="n">
         <f aca="false">J11/12*Supuestos!$D$9</f>
         <v>12000</v>
       </c>
-      <c r="T11" s="50" t="n">
+      <c r="T11" s="51" t="n">
         <f aca="false">K11/12*Supuestos!$D$9*Supuestos!$D$11</f>
         <v>0</v>
       </c>
-      <c r="U11" s="51" t="n">
+      <c r="U11" s="52" t="n">
         <f aca="false">SUM(O11:T11)</f>
         <v>226000</v>
       </c>
-      <c r="V11" s="52" t="s">
-        <v>140</v>
-      </c>
-      <c r="W11" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="X11" s="52" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y11" s="53" t="str">
+      <c r="V11" s="53" t="s">
+        <v>146</v>
+      </c>
+      <c r="W11" s="53" t="s">
+        <v>76</v>
+      </c>
+      <c r="X11" s="53" t="s">
+        <v>147</v>
+      </c>
+      <c r="Y11" s="54" t="str">
         <f aca="false">IF(X11="Automático",IF(W11="Caracas","Sí",IF(W11="Maracaibo","No",IF(W11="Otro","Sí","Por definir"))),X11)</f>
         <v>Por definir</v>
       </c>
-      <c r="Z11" s="45" t="n">
+      <c r="Z11" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="AA11" s="49" t="n">
-        <f aca="false">IF(V11="Expatriado",L11/12*Supuestos!$D$10,IF(V11="Repatriado",(F11+H11+J11+K11+IF(Y11="No",0,G11))/12*Supuestos!$D$10,0))</f>
+      <c r="AA11" s="50" t="n">
+        <f aca="false">IF(V11="Expatriado",(F11+G11+H11+I11+J11+K11*Supuestos!$D$13)/12*Supuestos!$D$10,IF(V11="Repatriado",(F11+H11+J11+K11*Supuestos!$D$12+IF(Y11="No",0,G11))/12*Supuestos!$D$10,0))</f>
         <v>262000</v>
       </c>
-      <c r="AB11" s="51" t="n">
+      <c r="AB11" s="52" t="n">
         <f aca="false">AA11+Z11</f>
         <v>262000</v>
       </c>
-      <c r="AC11" s="51" t="n">
+      <c r="AC11" s="52" t="n">
         <f aca="false">U11+AB11</f>
         <v>488000</v>
       </c>
-      <c r="AD11" s="48" t="n">
+      <c r="AD11" s="49" t="n">
         <f aca="false">M11-AC11</f>
         <v>36000</v>
       </c>
-      <c r="AE11" s="48" t="n">
-        <f aca="false">IF(V11="Expatriado",M11,IF(V11="Repatriado",F11+H11+J11+K11+IF(Y11="No",0,G11),0))</f>
+      <c r="AE11" s="49" t="n">
+        <f aca="false">IF(V11="Expatriado",F11+G11+H11+I11+J11+K11*Supuestos!$D$13,IF(V11="Repatriado",F11+H11+J11+K11*Supuestos!$D$12+IF(Y11="No",0,G11),0))</f>
         <v>524000</v>
       </c>
-      <c r="AF11" s="54" t="str">
+      <c r="AF11" s="55" t="str">
         <f aca="false">IF(V11="Por definir","Definir paquete",IF(W11="Por definir","Definir ciudad",IF(AND(V11="Repatriado",Y11="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C12" s="43" t="n">
+      <c r="C12" s="44" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="44" t="s">
-        <v>142</v>
-      </c>
-      <c r="E12" s="44" t="s">
-        <v>143</v>
-      </c>
-      <c r="F12" s="45" t="n">
+      <c r="D12" s="45" t="s">
+        <v>148</v>
+      </c>
+      <c r="E12" s="45" t="s">
+        <v>149</v>
+      </c>
+      <c r="F12" s="46" t="n">
         <v>216000</v>
       </c>
-      <c r="G12" s="46" t="n">
+      <c r="G12" s="47" t="n">
         <v>24000</v>
       </c>
-      <c r="H12" s="46" t="n">
+      <c r="H12" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="I12" s="46" t="n">
+      <c r="I12" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="J12" s="46" t="n">
+      <c r="J12" s="47" t="n">
         <v>18000</v>
       </c>
-      <c r="K12" s="46" t="n">
+      <c r="K12" s="47" t="n">
         <v>43200</v>
       </c>
-      <c r="L12" s="47" t="n">
+      <c r="L12" s="48" t="n">
         <f aca="false">SUM(F12:K12)</f>
         <v>325200</v>
       </c>
-      <c r="M12" s="46" t="n">
+      <c r="M12" s="47" t="n">
         <v>325200</v>
       </c>
-      <c r="N12" s="48" t="n">
+      <c r="N12" s="49" t="n">
         <f aca="false">L12-M12</f>
         <v>0</v>
       </c>
-      <c r="O12" s="49" t="n">
+      <c r="O12" s="50" t="n">
         <f aca="false">F12/12*Supuestos!$D$9</f>
         <v>108000</v>
       </c>
-      <c r="P12" s="50" t="n">
+      <c r="P12" s="51" t="n">
         <f aca="false">G12/12*Supuestos!$D$9</f>
         <v>12000</v>
       </c>
-      <c r="Q12" s="50" t="n">
+      <c r="Q12" s="51" t="n">
         <f aca="false">H12/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="R12" s="50" t="n">
+      <c r="R12" s="51" t="n">
         <f aca="false">I12/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="S12" s="50" t="n">
+      <c r="S12" s="51" t="n">
         <f aca="false">J12/12*Supuestos!$D$9</f>
         <v>9000</v>
       </c>
-      <c r="T12" s="50" t="n">
+      <c r="T12" s="51" t="n">
         <f aca="false">K12/12*Supuestos!$D$9*Supuestos!$D$11</f>
         <v>0</v>
       </c>
-      <c r="U12" s="51" t="n">
+      <c r="U12" s="52" t="n">
         <f aca="false">SUM(O12:T12)</f>
         <v>141000</v>
       </c>
-      <c r="V12" s="52" t="s">
-        <v>140</v>
-      </c>
-      <c r="W12" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="X12" s="52" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y12" s="53" t="str">
+      <c r="V12" s="53" t="s">
+        <v>146</v>
+      </c>
+      <c r="W12" s="53" t="s">
+        <v>76</v>
+      </c>
+      <c r="X12" s="53" t="s">
+        <v>147</v>
+      </c>
+      <c r="Y12" s="54" t="str">
         <f aca="false">IF(X12="Automático",IF(W12="Caracas","Sí",IF(W12="Maracaibo","No",IF(W12="Otro","Sí","Por definir"))),X12)</f>
         <v>Por definir</v>
       </c>
-      <c r="Z12" s="45" t="n">
+      <c r="Z12" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="AA12" s="49" t="n">
-        <f aca="false">IF(V12="Expatriado",L12/12*Supuestos!$D$10,IF(V12="Repatriado",(F12+H12+J12+K12+IF(Y12="No",0,G12))/12*Supuestos!$D$10,0))</f>
+      <c r="AA12" s="50" t="n">
+        <f aca="false">IF(V12="Expatriado",(F12+G12+H12+I12+J12+K12*Supuestos!$D$13)/12*Supuestos!$D$10,IF(V12="Repatriado",(F12+H12+J12+K12*Supuestos!$D$12+IF(Y12="No",0,G12))/12*Supuestos!$D$10,0))</f>
         <v>162600</v>
       </c>
-      <c r="AB12" s="51" t="n">
+      <c r="AB12" s="52" t="n">
         <f aca="false">AA12+Z12</f>
         <v>162600</v>
       </c>
-      <c r="AC12" s="51" t="n">
+      <c r="AC12" s="52" t="n">
         <f aca="false">U12+AB12</f>
         <v>303600</v>
       </c>
-      <c r="AD12" s="48" t="n">
+      <c r="AD12" s="49" t="n">
         <f aca="false">M12-AC12</f>
         <v>21600</v>
       </c>
-      <c r="AE12" s="48" t="n">
-        <f aca="false">IF(V12="Expatriado",M12,IF(V12="Repatriado",F12+H12+J12+K12+IF(Y12="No",0,G12),0))</f>
+      <c r="AE12" s="49" t="n">
+        <f aca="false">IF(V12="Expatriado",F12+G12+H12+I12+J12+K12*Supuestos!$D$13,IF(V12="Repatriado",F12+H12+J12+K12*Supuestos!$D$12+IF(Y12="No",0,G12),0))</f>
         <v>325200</v>
       </c>
-      <c r="AF12" s="54" t="str">
+      <c r="AF12" s="55" t="str">
         <f aca="false">IF(V12="Por definir","Definir paquete",IF(W12="Por definir","Definir ciudad",IF(AND(V12="Repatriado",Y12="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C13" s="43" t="n">
+      <c r="C13" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="D13" s="44" t="s">
-        <v>144</v>
-      </c>
-      <c r="E13" s="44" t="s">
-        <v>145</v>
-      </c>
-      <c r="F13" s="45" t="n">
+      <c r="D13" s="45" t="s">
+        <v>150</v>
+      </c>
+      <c r="E13" s="45" t="s">
+        <v>151</v>
+      </c>
+      <c r="F13" s="46" t="n">
         <v>180000</v>
       </c>
-      <c r="G13" s="46" t="n">
+      <c r="G13" s="47" t="n">
         <v>24000</v>
       </c>
-      <c r="H13" s="46" t="n">
+      <c r="H13" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="I13" s="46" t="n">
+      <c r="I13" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="J13" s="46" t="n">
+      <c r="J13" s="47" t="n">
         <v>18000</v>
       </c>
-      <c r="K13" s="46" t="n">
+      <c r="K13" s="47" t="n">
         <v>36000</v>
       </c>
-      <c r="L13" s="47" t="n">
+      <c r="L13" s="48" t="n">
         <f aca="false">SUM(F13:K13)</f>
         <v>282000</v>
       </c>
-      <c r="M13" s="46" t="n">
+      <c r="M13" s="47" t="n">
         <v>282000</v>
       </c>
-      <c r="N13" s="48" t="n">
+      <c r="N13" s="49" t="n">
         <f aca="false">L13-M13</f>
         <v>0</v>
       </c>
-      <c r="O13" s="49" t="n">
+      <c r="O13" s="50" t="n">
         <f aca="false">F13/12*Supuestos!$D$9</f>
         <v>90000</v>
       </c>
-      <c r="P13" s="50" t="n">
+      <c r="P13" s="51" t="n">
         <f aca="false">G13/12*Supuestos!$D$9</f>
         <v>12000</v>
       </c>
-      <c r="Q13" s="50" t="n">
+      <c r="Q13" s="51" t="n">
         <f aca="false">H13/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="R13" s="50" t="n">
+      <c r="R13" s="51" t="n">
         <f aca="false">I13/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="S13" s="50" t="n">
+      <c r="S13" s="51" t="n">
         <f aca="false">J13/12*Supuestos!$D$9</f>
         <v>9000</v>
       </c>
-      <c r="T13" s="50" t="n">
+      <c r="T13" s="51" t="n">
         <f aca="false">K13/12*Supuestos!$D$9*Supuestos!$D$11</f>
         <v>0</v>
       </c>
-      <c r="U13" s="51" t="n">
+      <c r="U13" s="52" t="n">
         <f aca="false">SUM(O13:T13)</f>
         <v>123000</v>
       </c>
-      <c r="V13" s="52" t="s">
-        <v>140</v>
-      </c>
-      <c r="W13" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="X13" s="52" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y13" s="53" t="str">
+      <c r="V13" s="53" t="s">
+        <v>146</v>
+      </c>
+      <c r="W13" s="53" t="s">
+        <v>76</v>
+      </c>
+      <c r="X13" s="53" t="s">
+        <v>147</v>
+      </c>
+      <c r="Y13" s="54" t="str">
         <f aca="false">IF(X13="Automático",IF(W13="Caracas","Sí",IF(W13="Maracaibo","No",IF(W13="Otro","Sí","Por definir"))),X13)</f>
         <v>Por definir</v>
       </c>
-      <c r="Z13" s="45" t="n">
+      <c r="Z13" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="AA13" s="49" t="n">
-        <f aca="false">IF(V13="Expatriado",L13/12*Supuestos!$D$10,IF(V13="Repatriado",(F13+H13+J13+K13+IF(Y13="No",0,G13))/12*Supuestos!$D$10,0))</f>
+      <c r="AA13" s="50" t="n">
+        <f aca="false">IF(V13="Expatriado",(F13+G13+H13+I13+J13+K13*Supuestos!$D$13)/12*Supuestos!$D$10,IF(V13="Repatriado",(F13+H13+J13+K13*Supuestos!$D$12+IF(Y13="No",0,G13))/12*Supuestos!$D$10,0))</f>
         <v>141000</v>
       </c>
-      <c r="AB13" s="51" t="n">
+      <c r="AB13" s="52" t="n">
         <f aca="false">AA13+Z13</f>
         <v>141000</v>
       </c>
-      <c r="AC13" s="51" t="n">
+      <c r="AC13" s="52" t="n">
         <f aca="false">U13+AB13</f>
         <v>264000</v>
       </c>
-      <c r="AD13" s="48" t="n">
+      <c r="AD13" s="49" t="n">
         <f aca="false">M13-AC13</f>
         <v>18000</v>
       </c>
-      <c r="AE13" s="48" t="n">
-        <f aca="false">IF(V13="Expatriado",M13,IF(V13="Repatriado",F13+H13+J13+K13+IF(Y13="No",0,G13),0))</f>
+      <c r="AE13" s="49" t="n">
+        <f aca="false">IF(V13="Expatriado",F13+G13+H13+I13+J13+K13*Supuestos!$D$13,IF(V13="Repatriado",F13+H13+J13+K13*Supuestos!$D$12+IF(Y13="No",0,G13),0))</f>
         <v>282000</v>
       </c>
-      <c r="AF13" s="54" t="str">
+      <c r="AF13" s="55" t="str">
         <f aca="false">IF(V13="Por definir","Definir paquete",IF(W13="Por definir","Definir ciudad",IF(AND(V13="Repatriado",Y13="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C14" s="43" t="n">
+      <c r="C14" s="44" t="n">
         <v>4</v>
       </c>
-      <c r="D14" s="44" t="s">
-        <v>146</v>
-      </c>
-      <c r="E14" s="44" t="s">
-        <v>147</v>
-      </c>
-      <c r="F14" s="45" t="n">
+      <c r="D14" s="45" t="s">
+        <v>152</v>
+      </c>
+      <c r="E14" s="45" t="s">
+        <v>153</v>
+      </c>
+      <c r="F14" s="46" t="n">
         <v>216000</v>
       </c>
-      <c r="G14" s="46" t="n">
+      <c r="G14" s="47" t="n">
         <v>24000</v>
       </c>
-      <c r="H14" s="46" t="n">
+      <c r="H14" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="I14" s="46" t="n">
+      <c r="I14" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="J14" s="46" t="n">
+      <c r="J14" s="47" t="n">
         <v>18000</v>
       </c>
-      <c r="K14" s="46" t="n">
+      <c r="K14" s="47" t="n">
         <v>43200</v>
       </c>
-      <c r="L14" s="47" t="n">
+      <c r="L14" s="48" t="n">
         <f aca="false">SUM(F14:K14)</f>
         <v>325200</v>
       </c>
-      <c r="M14" s="46" t="n">
+      <c r="M14" s="47" t="n">
         <v>325200</v>
       </c>
-      <c r="N14" s="48" t="n">
+      <c r="N14" s="49" t="n">
         <f aca="false">L14-M14</f>
         <v>0</v>
       </c>
-      <c r="O14" s="49" t="n">
+      <c r="O14" s="50" t="n">
         <f aca="false">F14/12*Supuestos!$D$9</f>
         <v>108000</v>
       </c>
-      <c r="P14" s="50" t="n">
+      <c r="P14" s="51" t="n">
         <f aca="false">G14/12*Supuestos!$D$9</f>
         <v>12000</v>
       </c>
-      <c r="Q14" s="50" t="n">
+      <c r="Q14" s="51" t="n">
         <f aca="false">H14/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="R14" s="50" t="n">
+      <c r="R14" s="51" t="n">
         <f aca="false">I14/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="S14" s="50" t="n">
+      <c r="S14" s="51" t="n">
         <f aca="false">J14/12*Supuestos!$D$9</f>
         <v>9000</v>
       </c>
-      <c r="T14" s="50" t="n">
+      <c r="T14" s="51" t="n">
         <f aca="false">K14/12*Supuestos!$D$9*Supuestos!$D$11</f>
         <v>0</v>
       </c>
-      <c r="U14" s="51" t="n">
+      <c r="U14" s="52" t="n">
         <f aca="false">SUM(O14:T14)</f>
         <v>141000</v>
       </c>
-      <c r="V14" s="52" t="s">
-        <v>140</v>
-      </c>
-      <c r="W14" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="X14" s="52" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y14" s="53" t="str">
+      <c r="V14" s="53" t="s">
+        <v>146</v>
+      </c>
+      <c r="W14" s="53" t="s">
+        <v>76</v>
+      </c>
+      <c r="X14" s="53" t="s">
+        <v>147</v>
+      </c>
+      <c r="Y14" s="54" t="str">
         <f aca="false">IF(X14="Automático",IF(W14="Caracas","Sí",IF(W14="Maracaibo","No",IF(W14="Otro","Sí","Por definir"))),X14)</f>
         <v>Por definir</v>
       </c>
-      <c r="Z14" s="45" t="n">
+      <c r="Z14" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="AA14" s="49" t="n">
-        <f aca="false">IF(V14="Expatriado",L14/12*Supuestos!$D$10,IF(V14="Repatriado",(F14+H14+J14+K14+IF(Y14="No",0,G14))/12*Supuestos!$D$10,0))</f>
+      <c r="AA14" s="50" t="n">
+        <f aca="false">IF(V14="Expatriado",(F14+G14+H14+I14+J14+K14*Supuestos!$D$13)/12*Supuestos!$D$10,IF(V14="Repatriado",(F14+H14+J14+K14*Supuestos!$D$12+IF(Y14="No",0,G14))/12*Supuestos!$D$10,0))</f>
         <v>162600</v>
       </c>
-      <c r="AB14" s="51" t="n">
+      <c r="AB14" s="52" t="n">
         <f aca="false">AA14+Z14</f>
         <v>162600</v>
       </c>
-      <c r="AC14" s="51" t="n">
+      <c r="AC14" s="52" t="n">
         <f aca="false">U14+AB14</f>
         <v>303600</v>
       </c>
-      <c r="AD14" s="48" t="n">
+      <c r="AD14" s="49" t="n">
         <f aca="false">M14-AC14</f>
         <v>21600</v>
       </c>
-      <c r="AE14" s="48" t="n">
-        <f aca="false">IF(V14="Expatriado",M14,IF(V14="Repatriado",F14+H14+J14+K14+IF(Y14="No",0,G14),0))</f>
+      <c r="AE14" s="49" t="n">
+        <f aca="false">IF(V14="Expatriado",F14+G14+H14+I14+J14+K14*Supuestos!$D$13,IF(V14="Repatriado",F14+H14+J14+K14*Supuestos!$D$12+IF(Y14="No",0,G14),0))</f>
         <v>325200</v>
       </c>
-      <c r="AF14" s="54" t="str">
+      <c r="AF14" s="55" t="str">
         <f aca="false">IF(V14="Por definir","Definir paquete",IF(W14="Por definir","Definir ciudad",IF(AND(V14="Repatriado",Y14="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C15" s="43" t="n">
+      <c r="C15" s="44" t="n">
         <v>5</v>
       </c>
-      <c r="D15" s="44" t="s">
-        <v>148</v>
-      </c>
-      <c r="E15" s="44" t="s">
-        <v>149</v>
-      </c>
-      <c r="F15" s="45" t="n">
+      <c r="D15" s="45" t="s">
+        <v>154</v>
+      </c>
+      <c r="E15" s="45" t="s">
+        <v>155</v>
+      </c>
+      <c r="F15" s="46" t="n">
         <v>180000</v>
       </c>
-      <c r="G15" s="46" t="n">
+      <c r="G15" s="47" t="n">
         <v>24000</v>
       </c>
-      <c r="H15" s="46" t="n">
+      <c r="H15" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="I15" s="46" t="n">
+      <c r="I15" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="J15" s="46" t="n">
+      <c r="J15" s="47" t="n">
         <v>18000</v>
       </c>
-      <c r="K15" s="46" t="n">
+      <c r="K15" s="47" t="n">
         <v>36000</v>
       </c>
-      <c r="L15" s="47" t="n">
+      <c r="L15" s="48" t="n">
         <f aca="false">SUM(F15:K15)</f>
         <v>282000</v>
       </c>
-      <c r="M15" s="46" t="n">
+      <c r="M15" s="47" t="n">
         <v>282000</v>
       </c>
-      <c r="N15" s="48" t="n">
+      <c r="N15" s="49" t="n">
         <f aca="false">L15-M15</f>
         <v>0</v>
       </c>
-      <c r="O15" s="49" t="n">
+      <c r="O15" s="50" t="n">
         <f aca="false">F15/12*Supuestos!$D$9</f>
         <v>90000</v>
       </c>
-      <c r="P15" s="50" t="n">
+      <c r="P15" s="51" t="n">
         <f aca="false">G15/12*Supuestos!$D$9</f>
         <v>12000</v>
       </c>
-      <c r="Q15" s="50" t="n">
+      <c r="Q15" s="51" t="n">
         <f aca="false">H15/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="R15" s="50" t="n">
+      <c r="R15" s="51" t="n">
         <f aca="false">I15/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="S15" s="50" t="n">
+      <c r="S15" s="51" t="n">
         <f aca="false">J15/12*Supuestos!$D$9</f>
         <v>9000</v>
       </c>
-      <c r="T15" s="50" t="n">
+      <c r="T15" s="51" t="n">
         <f aca="false">K15/12*Supuestos!$D$9*Supuestos!$D$11</f>
         <v>0</v>
       </c>
-      <c r="U15" s="51" t="n">
+      <c r="U15" s="52" t="n">
         <f aca="false">SUM(O15:T15)</f>
         <v>123000</v>
       </c>
-      <c r="V15" s="52" t="s">
-        <v>140</v>
-      </c>
-      <c r="W15" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="X15" s="52" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y15" s="53" t="str">
+      <c r="V15" s="53" t="s">
+        <v>146</v>
+      </c>
+      <c r="W15" s="53" t="s">
+        <v>76</v>
+      </c>
+      <c r="X15" s="53" t="s">
+        <v>147</v>
+      </c>
+      <c r="Y15" s="54" t="str">
         <f aca="false">IF(X15="Automático",IF(W15="Caracas","Sí",IF(W15="Maracaibo","No",IF(W15="Otro","Sí","Por definir"))),X15)</f>
         <v>Por definir</v>
       </c>
-      <c r="Z15" s="45" t="n">
+      <c r="Z15" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="AA15" s="49" t="n">
-        <f aca="false">IF(V15="Expatriado",L15/12*Supuestos!$D$10,IF(V15="Repatriado",(F15+H15+J15+K15+IF(Y15="No",0,G15))/12*Supuestos!$D$10,0))</f>
+      <c r="AA15" s="50" t="n">
+        <f aca="false">IF(V15="Expatriado",(F15+G15+H15+I15+J15+K15*Supuestos!$D$13)/12*Supuestos!$D$10,IF(V15="Repatriado",(F15+H15+J15+K15*Supuestos!$D$12+IF(Y15="No",0,G15))/12*Supuestos!$D$10,0))</f>
         <v>141000</v>
       </c>
-      <c r="AB15" s="51" t="n">
+      <c r="AB15" s="52" t="n">
         <f aca="false">AA15+Z15</f>
         <v>141000</v>
       </c>
-      <c r="AC15" s="51" t="n">
+      <c r="AC15" s="52" t="n">
         <f aca="false">U15+AB15</f>
         <v>264000</v>
       </c>
-      <c r="AD15" s="48" t="n">
+      <c r="AD15" s="49" t="n">
         <f aca="false">M15-AC15</f>
         <v>18000</v>
       </c>
-      <c r="AE15" s="48" t="n">
-        <f aca="false">IF(V15="Expatriado",M15,IF(V15="Repatriado",F15+H15+J15+K15+IF(Y15="No",0,G15),0))</f>
+      <c r="AE15" s="49" t="n">
+        <f aca="false">IF(V15="Expatriado",F15+G15+H15+I15+J15+K15*Supuestos!$D$13,IF(V15="Repatriado",F15+H15+J15+K15*Supuestos!$D$12+IF(Y15="No",0,G15),0))</f>
         <v>282000</v>
       </c>
-      <c r="AF15" s="54" t="str">
+      <c r="AF15" s="55" t="str">
         <f aca="false">IF(V15="Por definir","Definir paquete",IF(W15="Por definir","Definir ciudad",IF(AND(V15="Repatriado",Y15="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C16" s="43" t="n">
+      <c r="C16" s="44" t="n">
         <v>6</v>
       </c>
-      <c r="D16" s="44" t="s">
-        <v>150</v>
-      </c>
-      <c r="E16" s="44" t="s">
-        <v>151</v>
-      </c>
-      <c r="F16" s="45" t="n">
+      <c r="D16" s="45" t="s">
+        <v>156</v>
+      </c>
+      <c r="E16" s="45" t="s">
+        <v>157</v>
+      </c>
+      <c r="F16" s="46" t="n">
         <v>120000</v>
       </c>
-      <c r="G16" s="46" t="n">
+      <c r="G16" s="47" t="n">
         <v>18000</v>
       </c>
-      <c r="H16" s="46" t="n">
+      <c r="H16" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="I16" s="46" t="n">
+      <c r="I16" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="J16" s="46" t="n">
+      <c r="J16" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="K16" s="46" t="n">
+      <c r="K16" s="47" t="n">
         <v>20000</v>
       </c>
-      <c r="L16" s="47" t="n">
+      <c r="L16" s="48" t="n">
         <f aca="false">SUM(F16:K16)</f>
         <v>194000</v>
       </c>
-      <c r="M16" s="46" t="n">
+      <c r="M16" s="47" t="n">
         <v>194000</v>
       </c>
-      <c r="N16" s="48" t="n">
+      <c r="N16" s="49" t="n">
         <f aca="false">L16-M16</f>
         <v>0</v>
       </c>
-      <c r="O16" s="49" t="n">
+      <c r="O16" s="50" t="n">
         <f aca="false">F16/12*Supuestos!$D$9</f>
         <v>60000</v>
       </c>
-      <c r="P16" s="50" t="n">
+      <c r="P16" s="51" t="n">
         <f aca="false">G16/12*Supuestos!$D$9</f>
         <v>9000</v>
       </c>
-      <c r="Q16" s="50" t="n">
+      <c r="Q16" s="51" t="n">
         <f aca="false">H16/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="R16" s="50" t="n">
+      <c r="R16" s="51" t="n">
         <f aca="false">I16/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="S16" s="50" t="n">
+      <c r="S16" s="51" t="n">
         <f aca="false">J16/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="T16" s="50" t="n">
+      <c r="T16" s="51" t="n">
         <f aca="false">K16/12*Supuestos!$D$9*Supuestos!$D$11</f>
         <v>0</v>
       </c>
-      <c r="U16" s="51" t="n">
+      <c r="U16" s="52" t="n">
         <f aca="false">SUM(O16:T16)</f>
         <v>87000</v>
       </c>
-      <c r="V16" s="52" t="s">
-        <v>140</v>
-      </c>
-      <c r="W16" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="X16" s="52" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y16" s="53" t="str">
+      <c r="V16" s="53" t="s">
+        <v>146</v>
+      </c>
+      <c r="W16" s="53" t="s">
+        <v>76</v>
+      </c>
+      <c r="X16" s="53" t="s">
+        <v>147</v>
+      </c>
+      <c r="Y16" s="54" t="str">
         <f aca="false">IF(X16="Automático",IF(W16="Caracas","Sí",IF(W16="Maracaibo","No",IF(W16="Otro","Sí","Por definir"))),X16)</f>
         <v>Por definir</v>
       </c>
-      <c r="Z16" s="45" t="n">
+      <c r="Z16" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="AA16" s="49" t="n">
-        <f aca="false">IF(V16="Expatriado",L16/12*Supuestos!$D$10,IF(V16="Repatriado",(F16+H16+J16+K16+IF(Y16="No",0,G16))/12*Supuestos!$D$10,0))</f>
+      <c r="AA16" s="50" t="n">
+        <f aca="false">IF(V16="Expatriado",(F16+G16+H16+I16+J16+K16*Supuestos!$D$13)/12*Supuestos!$D$10,IF(V16="Repatriado",(F16+H16+J16+K16*Supuestos!$D$12+IF(Y16="No",0,G16))/12*Supuestos!$D$10,0))</f>
         <v>97000</v>
       </c>
-      <c r="AB16" s="51" t="n">
+      <c r="AB16" s="52" t="n">
         <f aca="false">AA16+Z16</f>
         <v>97000</v>
       </c>
-      <c r="AC16" s="51" t="n">
+      <c r="AC16" s="52" t="n">
         <f aca="false">U16+AB16</f>
         <v>184000</v>
       </c>
-      <c r="AD16" s="48" t="n">
+      <c r="AD16" s="49" t="n">
         <f aca="false">M16-AC16</f>
         <v>10000</v>
       </c>
-      <c r="AE16" s="48" t="n">
-        <f aca="false">IF(V16="Expatriado",M16,IF(V16="Repatriado",F16+H16+J16+K16+IF(Y16="No",0,G16),0))</f>
+      <c r="AE16" s="49" t="n">
+        <f aca="false">IF(V16="Expatriado",F16+G16+H16+I16+J16+K16*Supuestos!$D$13,IF(V16="Repatriado",F16+H16+J16+K16*Supuestos!$D$12+IF(Y16="No",0,G16),0))</f>
         <v>194000</v>
       </c>
-      <c r="AF16" s="54" t="str">
+      <c r="AF16" s="55" t="str">
         <f aca="false">IF(V16="Por definir","Definir paquete",IF(W16="Por definir","Definir ciudad",IF(AND(V16="Repatriado",Y16="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C17" s="43" t="n">
+      <c r="C17" s="44" t="n">
         <v>7</v>
       </c>
-      <c r="D17" s="44" t="s">
-        <v>152</v>
-      </c>
-      <c r="E17" s="44" t="s">
-        <v>153</v>
-      </c>
-      <c r="F17" s="45" t="n">
+      <c r="D17" s="45" t="s">
+        <v>158</v>
+      </c>
+      <c r="E17" s="45" t="s">
+        <v>159</v>
+      </c>
+      <c r="F17" s="46" t="n">
         <v>180000</v>
       </c>
-      <c r="G17" s="46" t="n">
+      <c r="G17" s="47" t="n">
         <v>24000</v>
       </c>
-      <c r="H17" s="46" t="n">
+      <c r="H17" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="I17" s="46" t="n">
+      <c r="I17" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="J17" s="46" t="n">
+      <c r="J17" s="47" t="n">
         <v>18000</v>
       </c>
-      <c r="K17" s="46" t="n">
+      <c r="K17" s="47" t="n">
         <v>36000</v>
       </c>
-      <c r="L17" s="47" t="n">
+      <c r="L17" s="48" t="n">
         <f aca="false">SUM(F17:K17)</f>
         <v>282000</v>
       </c>
-      <c r="M17" s="46" t="n">
+      <c r="M17" s="47" t="n">
         <v>282000</v>
       </c>
-      <c r="N17" s="48" t="n">
+      <c r="N17" s="49" t="n">
         <f aca="false">L17-M17</f>
         <v>0</v>
       </c>
-      <c r="O17" s="49" t="n">
+      <c r="O17" s="50" t="n">
         <f aca="false">F17/12*Supuestos!$D$9</f>
         <v>90000</v>
       </c>
-      <c r="P17" s="50" t="n">
+      <c r="P17" s="51" t="n">
         <f aca="false">G17/12*Supuestos!$D$9</f>
         <v>12000</v>
       </c>
-      <c r="Q17" s="50" t="n">
+      <c r="Q17" s="51" t="n">
         <f aca="false">H17/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="R17" s="50" t="n">
+      <c r="R17" s="51" t="n">
         <f aca="false">I17/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="S17" s="50" t="n">
+      <c r="S17" s="51" t="n">
         <f aca="false">J17/12*Supuestos!$D$9</f>
         <v>9000</v>
       </c>
-      <c r="T17" s="50" t="n">
+      <c r="T17" s="51" t="n">
         <f aca="false">K17/12*Supuestos!$D$9*Supuestos!$D$11</f>
         <v>0</v>
       </c>
-      <c r="U17" s="51" t="n">
+      <c r="U17" s="52" t="n">
         <f aca="false">SUM(O17:T17)</f>
         <v>123000</v>
       </c>
-      <c r="V17" s="52" t="s">
-        <v>140</v>
-      </c>
-      <c r="W17" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="X17" s="52" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y17" s="53" t="str">
+      <c r="V17" s="53" t="s">
+        <v>146</v>
+      </c>
+      <c r="W17" s="53" t="s">
+        <v>76</v>
+      </c>
+      <c r="X17" s="53" t="s">
+        <v>147</v>
+      </c>
+      <c r="Y17" s="54" t="str">
         <f aca="false">IF(X17="Automático",IF(W17="Caracas","Sí",IF(W17="Maracaibo","No",IF(W17="Otro","Sí","Por definir"))),X17)</f>
         <v>Por definir</v>
       </c>
-      <c r="Z17" s="45" t="n">
+      <c r="Z17" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="AA17" s="49" t="n">
-        <f aca="false">IF(V17="Expatriado",L17/12*Supuestos!$D$10,IF(V17="Repatriado",(F17+H17+J17+K17+IF(Y17="No",0,G17))/12*Supuestos!$D$10,0))</f>
+      <c r="AA17" s="50" t="n">
+        <f aca="false">IF(V17="Expatriado",(F17+G17+H17+I17+J17+K17*Supuestos!$D$13)/12*Supuestos!$D$10,IF(V17="Repatriado",(F17+H17+J17+K17*Supuestos!$D$12+IF(Y17="No",0,G17))/12*Supuestos!$D$10,0))</f>
         <v>141000</v>
       </c>
-      <c r="AB17" s="51" t="n">
+      <c r="AB17" s="52" t="n">
         <f aca="false">AA17+Z17</f>
         <v>141000</v>
       </c>
-      <c r="AC17" s="51" t="n">
+      <c r="AC17" s="52" t="n">
         <f aca="false">U17+AB17</f>
         <v>264000</v>
       </c>
-      <c r="AD17" s="48" t="n">
+      <c r="AD17" s="49" t="n">
         <f aca="false">M17-AC17</f>
         <v>18000</v>
       </c>
-      <c r="AE17" s="48" t="n">
-        <f aca="false">IF(V17="Expatriado",M17,IF(V17="Repatriado",F17+H17+J17+K17+IF(Y17="No",0,G17),0))</f>
+      <c r="AE17" s="49" t="n">
+        <f aca="false">IF(V17="Expatriado",F17+G17+H17+I17+J17+K17*Supuestos!$D$13,IF(V17="Repatriado",F17+H17+J17+K17*Supuestos!$D$12+IF(Y17="No",0,G17),0))</f>
         <v>282000</v>
       </c>
-      <c r="AF17" s="54" t="str">
+      <c r="AF17" s="55" t="str">
         <f aca="false">IF(V17="Por definir","Definir paquete",IF(W17="Por definir","Definir ciudad",IF(AND(V17="Repatriado",Y17="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C18" s="43" t="n">
+      <c r="C18" s="44" t="n">
         <v>8</v>
       </c>
-      <c r="D18" s="44" t="s">
-        <v>154</v>
-      </c>
-      <c r="E18" s="44" t="s">
-        <v>155</v>
-      </c>
-      <c r="F18" s="45" t="n">
+      <c r="D18" s="45" t="s">
+        <v>160</v>
+      </c>
+      <c r="E18" s="45" t="s">
+        <v>161</v>
+      </c>
+      <c r="F18" s="46" t="n">
         <v>48000</v>
       </c>
-      <c r="G18" s="46" t="n">
+      <c r="G18" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="H18" s="46" t="n">
+      <c r="H18" s="47" t="n">
         <v>8000</v>
       </c>
-      <c r="I18" s="46" t="n">
+      <c r="I18" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="J18" s="46" t="n">
+      <c r="J18" s="47" t="n">
         <v>7200</v>
       </c>
-      <c r="K18" s="46" t="n">
+      <c r="K18" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="L18" s="47" t="n">
+      <c r="L18" s="48" t="n">
         <f aca="false">SUM(F18:K18)</f>
         <v>87200</v>
       </c>
-      <c r="M18" s="46" t="n">
+      <c r="M18" s="47" t="n">
         <v>87200</v>
       </c>
-      <c r="N18" s="48" t="n">
+      <c r="N18" s="49" t="n">
         <f aca="false">L18-M18</f>
         <v>0</v>
       </c>
-      <c r="O18" s="49" t="n">
+      <c r="O18" s="50" t="n">
         <f aca="false">F18/12*Supuestos!$D$9</f>
         <v>24000</v>
       </c>
-      <c r="P18" s="50" t="n">
+      <c r="P18" s="51" t="n">
         <f aca="false">G18/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="Q18" s="50" t="n">
+      <c r="Q18" s="51" t="n">
         <f aca="false">H18/12*Supuestos!$D$9</f>
         <v>4000</v>
       </c>
-      <c r="R18" s="50" t="n">
+      <c r="R18" s="51" t="n">
         <f aca="false">I18/12*Supuestos!$D$9</f>
         <v>0</v>
       </c>
-      <c r="S18" s="50" t="n">
+      <c r="S18" s="51" t="n">
         <f aca="false">J18/12*Supuestos!$D$9</f>
         <v>3600</v>
       </c>
-      <c r="T18" s="50" t="n">
+      <c r="T18" s="51" t="n">
         <f aca="false">K18/12*Supuestos!$D$9*Supuestos!$D$11</f>
         <v>0</v>
       </c>
-      <c r="U18" s="51" t="n">
+      <c r="U18" s="52" t="n">
         <f aca="false">SUM(O18:T18)</f>
         <v>37600</v>
       </c>
-      <c r="V18" s="52" t="s">
-        <v>140</v>
-      </c>
-      <c r="W18" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="X18" s="52" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y18" s="53" t="str">
+      <c r="V18" s="53" t="s">
+        <v>146</v>
+      </c>
+      <c r="W18" s="53" t="s">
+        <v>76</v>
+      </c>
+      <c r="X18" s="53" t="s">
+        <v>147</v>
+      </c>
+      <c r="Y18" s="54" t="str">
         <f aca="false">IF(X18="Automático",IF(W18="Caracas","Sí",IF(W18="Maracaibo","No",IF(W18="Otro","Sí","Por definir"))),X18)</f>
         <v>Por definir</v>
       </c>
-      <c r="Z18" s="45" t="n">
+      <c r="Z18" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="AA18" s="49" t="n">
-        <f aca="false">IF(V18="Expatriado",L18/12*Supuestos!$D$10,IF(V18="Repatriado",(F18+H18+J18+K18+IF(Y18="No",0,G18))/12*Supuestos!$D$10,0))</f>
+      <c r="AA18" s="50" t="n">
+        <f aca="false">IF(V18="Expatriado",(F18+G18+H18+I18+J18+K18*Supuestos!$D$13)/12*Supuestos!$D$10,IF(V18="Repatriado",(F18+H18+J18+K18*Supuestos!$D$12+IF(Y18="No",0,G18))/12*Supuestos!$D$10,0))</f>
         <v>43600</v>
       </c>
-      <c r="AB18" s="51" t="n">
+      <c r="AB18" s="52" t="n">
         <f aca="false">AA18+Z18</f>
         <v>43600</v>
       </c>
-      <c r="AC18" s="51" t="n">
+      <c r="AC18" s="52" t="n">
         <f aca="false">U18+AB18</f>
         <v>81200</v>
       </c>
-      <c r="AD18" s="48" t="n">
+      <c r="AD18" s="49" t="n">
         <f aca="false">M18-AC18</f>
         <v>6000</v>
       </c>
-      <c r="AE18" s="48" t="n">
-        <f aca="false">IF(V18="Expatriado",M18,IF(V18="Repatriado",F18+H18+J18+K18+IF(Y18="No",0,G18),0))</f>
+      <c r="AE18" s="49" t="n">
+        <f aca="false">IF(V18="Expatriado",F18+G18+H18+I18+J18+K18*Supuestos!$D$13,IF(V18="Repatriado",F18+H18+J18+K18*Supuestos!$D$12+IF(Y18="No",0,G18),0))</f>
         <v>87200</v>
       </c>
-      <c r="AF18" s="54" t="str">
+      <c r="AF18" s="55" t="str">
         <f aca="false">IF(V18="Por definir","Definir paquete",IF(W18="Por definir","Definir ciudad",IF(AND(V18="Repatriado",Y18="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C19" s="43" t="n">
+      <c r="C19" s="44" t="n">
         <v>9</v>
       </c>
-      <c r="D19" s="44" t="s">
-        <v>156</v>
-      </c>
-      <c r="E19" s="44" t="s">
-        <v>157</v>
-      </c>
-      <c r="F19" s="45" t="n">
+      <c r="D19" s="45" t="s">
+        <v>162</v>
+      </c>
+      <c r="E19" s="45" t="s">
+        <v>163</v>
+      </c>
+      <c r="F19" s="46" t="n">
         <v>48000</v>
       </c>
-      <c r="G19" s="46" t="n">
+      <c r="G19" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="H19" s="46" t="n">
+      <c r="H19" s="47" t="n">
         <v>8000</v>
       </c>
-      <c r="I19" s="46" t="n">
+      <c r="I19" s="47" t="n">
         <v>12000</v>
       </c>
-      <c r="J19" s="46" t="n">
+      <c r="J19" s="47" t="n">
         <v>7200</v>
       </c>
-      <c r="K19" s="46" t="n">
+      <c r="K19" s="47" t="n">
         <v>8000</v>
       </c>
-      <c r="L19" s="47" t="n">
+      <c r="L19" s="48" t="n">
         <f aca="false">SUM(F19:K19)</f>
         <v>95200</v>
       </c>
-      <c r="M19" s="46" t="n">
+      <c r="M19" s="47" t="n">
         <v>95200</v>
       </c>
-      <c r="N19" s="48" t="n">
+      <c r="N19" s="49" t="n">
         <f aca="false">L19-M19</f>
         <v>0</v>
       </c>
-      <c r="O19" s="49" t="n">
+      <c r="O19" s="50" t="n">
         <f aca="false">F19/12*Supuestos!$D$9</f>
         <v>24000</v>
       </c>
-      <c r="P19" s="50" t="n">
+      <c r="P19" s="51" t="n">
         <f aca="false">G19/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="Q19" s="50" t="n">
+      <c r="Q19" s="51" t="n">
         <f aca="false">H19/12*Supuestos!$D$9</f>
         <v>4000</v>
       </c>
-      <c r="R19" s="50" t="n">
+      <c r="R19" s="51" t="n">
         <f aca="false">I19/12*Supuestos!$D$9</f>
         <v>6000</v>
       </c>
-      <c r="S19" s="50" t="n">
+      <c r="S19" s="51" t="n">
         <f aca="false">J19/12*Supuestos!$D$9</f>
         <v>3600</v>
       </c>
-      <c r="T19" s="50" t="n">
+      <c r="T19" s="51" t="n">
         <f aca="false">K19/12*Supuestos!$D$9*Supuestos!$D$11</f>
         <v>0</v>
       </c>
-      <c r="U19" s="51" t="n">
+      <c r="U19" s="52" t="n">
         <f aca="false">SUM(O19:T19)</f>
         <v>43600</v>
       </c>
-      <c r="V19" s="52" t="s">
-        <v>140</v>
-      </c>
-      <c r="W19" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="X19" s="52" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y19" s="53" t="str">
+      <c r="V19" s="53" t="s">
+        <v>146</v>
+      </c>
+      <c r="W19" s="53" t="s">
+        <v>76</v>
+      </c>
+      <c r="X19" s="53" t="s">
+        <v>147</v>
+      </c>
+      <c r="Y19" s="54" t="str">
         <f aca="false">IF(X19="Automático",IF(W19="Caracas","Sí",IF(W19="Maracaibo","No",IF(W19="Otro","Sí","Por definir"))),X19)</f>
         <v>Por definir</v>
       </c>
-      <c r="Z19" s="45" t="n">
+      <c r="Z19" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="AA19" s="49" t="n">
-        <f aca="false">IF(V19="Expatriado",L19/12*Supuestos!$D$10,IF(V19="Repatriado",(F19+H19+J19+K19+IF(Y19="No",0,G19))/12*Supuestos!$D$10,0))</f>
+      <c r="AA19" s="50" t="n">
+        <f aca="false">IF(V19="Expatriado",(F19+G19+H19+I19+J19+K19*Supuestos!$D$13)/12*Supuestos!$D$10,IF(V19="Repatriado",(F19+H19+J19+K19*Supuestos!$D$12+IF(Y19="No",0,G19))/12*Supuestos!$D$10,0))</f>
         <v>47600</v>
       </c>
-      <c r="AB19" s="51" t="n">
+      <c r="AB19" s="52" t="n">
         <f aca="false">AA19+Z19</f>
         <v>47600</v>
       </c>
-      <c r="AC19" s="51" t="n">
+      <c r="AC19" s="52" t="n">
         <f aca="false">U19+AB19</f>
         <v>91200</v>
       </c>
-      <c r="AD19" s="48" t="n">
+      <c r="AD19" s="49" t="n">
         <f aca="false">M19-AC19</f>
         <v>4000</v>
       </c>
-      <c r="AE19" s="48" t="n">
-        <f aca="false">IF(V19="Expatriado",M19,IF(V19="Repatriado",F19+H19+J19+K19+IF(Y19="No",0,G19),0))</f>
+      <c r="AE19" s="49" t="n">
+        <f aca="false">IF(V19="Expatriado",F19+G19+H19+I19+J19+K19*Supuestos!$D$13,IF(V19="Repatriado",F19+H19+J19+K19*Supuestos!$D$12+IF(Y19="No",0,G19),0))</f>
         <v>95200</v>
       </c>
-      <c r="AF19" s="54" t="str">
+      <c r="AF19" s="55" t="str">
         <f aca="false">IF(V19="Por definir","Definir paquete",IF(W19="Por definir","Definir ciudad",IF(AND(V19="Repatriado",Y19="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C21" s="55"/>
-      <c r="D21" s="56" t="s">
-        <v>158</v>
-      </c>
-      <c r="E21" s="56"/>
-      <c r="F21" s="57" t="n">
+      <c r="C21" s="56"/>
+      <c r="D21" s="57" t="s">
+        <v>164</v>
+      </c>
+      <c r="E21" s="57"/>
+      <c r="F21" s="58" t="n">
         <f aca="false">SUM(F11:F19)</f>
         <v>1548000</v>
       </c>
-      <c r="G21" s="58" t="n">
+      <c r="G21" s="59" t="n">
         <f aca="false">SUM(G11:G19)</f>
         <v>198000</v>
       </c>
-      <c r="H21" s="58" t="n">
+      <c r="H21" s="59" t="n">
         <f aca="false">SUM(H11:H19)</f>
         <v>100000</v>
       </c>
-      <c r="I21" s="58" t="n">
+      <c r="I21" s="59" t="n">
         <f aca="false">SUM(I11:I19)</f>
         <v>104000</v>
       </c>
-      <c r="J21" s="58" t="n">
+      <c r="J21" s="59" t="n">
         <f aca="false">SUM(J11:J19)</f>
         <v>140400</v>
       </c>
-      <c r="K21" s="58" t="n">
+      <c r="K21" s="59" t="n">
         <f aca="false">SUM(K11:K19)</f>
         <v>306400</v>
       </c>
-      <c r="L21" s="58" t="n">
+      <c r="L21" s="59" t="n">
         <f aca="false">SUM(L11:L19)</f>
         <v>2396800</v>
       </c>
-      <c r="M21" s="58" t="n">
+      <c r="M21" s="59" t="n">
         <f aca="false">SUM(M11:M19)</f>
         <v>2396800</v>
       </c>
-      <c r="N21" s="58" t="n">
+      <c r="N21" s="59" t="n">
         <f aca="false">SUM(N11:N19)</f>
         <v>0</v>
       </c>
-      <c r="O21" s="57" t="n">
+      <c r="O21" s="58" t="n">
         <f aca="false">SUM(O11:O19)</f>
         <v>774000</v>
       </c>
-      <c r="P21" s="58" t="n">
+      <c r="P21" s="59" t="n">
         <f aca="false">SUM(P11:P19)</f>
         <v>99000</v>
       </c>
-      <c r="Q21" s="58" t="n">
+      <c r="Q21" s="59" t="n">
         <f aca="false">SUM(Q11:Q19)</f>
         <v>50000</v>
       </c>
-      <c r="R21" s="58" t="n">
+      <c r="R21" s="59" t="n">
         <f aca="false">SUM(R11:R19)</f>
         <v>52000</v>
       </c>
-      <c r="S21" s="58" t="n">
+      <c r="S21" s="59" t="n">
         <f aca="false">SUM(S11:S19)</f>
         <v>70200</v>
       </c>
-      <c r="T21" s="58" t="n">
+      <c r="T21" s="59" t="n">
         <f aca="false">SUM(T11:T19)</f>
         <v>0</v>
       </c>
-      <c r="U21" s="58" t="n">
+      <c r="U21" s="59" t="n">
         <f aca="false">SUM(U11:U19)</f>
         <v>1045200</v>
       </c>
-      <c r="V21" s="55"/>
-      <c r="W21" s="55"/>
-      <c r="X21" s="55"/>
-      <c r="Y21" s="55"/>
-      <c r="Z21" s="57" t="n">
+      <c r="V21" s="56"/>
+      <c r="W21" s="56"/>
+      <c r="X21" s="56"/>
+      <c r="Y21" s="56"/>
+      <c r="Z21" s="58" t="n">
         <f aca="false">SUM(Z11:Z19)</f>
         <v>0</v>
       </c>
-      <c r="AA21" s="58" t="n">
+      <c r="AA21" s="59" t="n">
         <f aca="false">SUM(AA11:AA19)</f>
         <v>1198400</v>
       </c>
-      <c r="AB21" s="58" t="n">
+      <c r="AB21" s="59" t="n">
         <f aca="false">SUM(AB11:AB19)</f>
         <v>1198400</v>
       </c>
-      <c r="AC21" s="58" t="n">
+      <c r="AC21" s="59" t="n">
         <f aca="false">SUM(AC11:AC19)</f>
         <v>2243600</v>
       </c>
-      <c r="AD21" s="58" t="n">
+      <c r="AD21" s="59" t="n">
         <f aca="false">SUM(AD11:AD19)</f>
         <v>153200</v>
       </c>
-      <c r="AE21" s="58" t="n">
+      <c r="AE21" s="59" t="n">
         <f aca="false">SUM(AE11:AE19)</f>
         <v>2396800</v>
       </c>
-      <c r="AF21" s="55"/>
+      <c r="AF21" s="56"/>
     </row>
   </sheetData>
   <autoFilter ref="C10:AF19"/>
@@ -8621,6 +8820,1187 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
+  <dimension ref="C3:T29"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="18" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="30"/>
+  </cols>
+  <sheetData>
+    <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C3" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
+      <c r="S3" s="1"/>
+      <c r="T3" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C5" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C6" s="3" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C8" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="4"/>
+      <c r="T8" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C10" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="N10" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="O10" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="P10" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q10" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="R10" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="S10" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="T10" s="5" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C11" s="26" t="str">
+        <f aca="false">Personal!E11</f>
+        <v>Martin del Castillo</v>
+      </c>
+      <c r="D11" s="26" t="str">
+        <f aca="false">Personal!D11</f>
+        <v>COO / PU General Manager</v>
+      </c>
+      <c r="E11" s="26" t="str">
+        <f aca="false">Personal!V11</f>
+        <v>Expatriado</v>
+      </c>
+      <c r="F11" s="26" t="str">
+        <f aca="false">Personal!W11</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G11" s="27" t="n">
+        <f aca="false">Personal!U11/Supuestos!$D$9</f>
+        <v>37666.6666666667</v>
+      </c>
+      <c r="H11" s="28" t="n">
+        <f aca="false">Personal!U11/Supuestos!$D$9</f>
+        <v>37666.6666666667</v>
+      </c>
+      <c r="I11" s="28" t="n">
+        <f aca="false">Personal!U11/Supuestos!$D$9</f>
+        <v>37666.6666666667</v>
+      </c>
+      <c r="J11" s="28" t="n">
+        <f aca="false">Personal!U11/Supuestos!$D$9</f>
+        <v>37666.6666666667</v>
+      </c>
+      <c r="K11" s="28" t="n">
+        <f aca="false">Personal!U11/Supuestos!$D$9</f>
+        <v>37666.6666666667</v>
+      </c>
+      <c r="L11" s="28" t="n">
+        <f aca="false">Personal!U11/Supuestos!$D$9</f>
+        <v>37666.6666666667</v>
+      </c>
+      <c r="M11" s="28" t="n">
+        <f aca="false">Personal!AA11/Supuestos!$D$10+Personal!Z11</f>
+        <v>43666.6666666667</v>
+      </c>
+      <c r="N11" s="28" t="n">
+        <f aca="false">Personal!AA11/Supuestos!$D$10</f>
+        <v>43666.6666666667</v>
+      </c>
+      <c r="O11" s="28" t="n">
+        <f aca="false">Personal!AA11/Supuestos!$D$10</f>
+        <v>43666.6666666667</v>
+      </c>
+      <c r="P11" s="28" t="n">
+        <f aca="false">Personal!AA11/Supuestos!$D$10</f>
+        <v>43666.6666666667</v>
+      </c>
+      <c r="Q11" s="28" t="n">
+        <f aca="false">Personal!AA11/Supuestos!$D$10</f>
+        <v>43666.6666666667</v>
+      </c>
+      <c r="R11" s="28" t="n">
+        <f aca="false">Personal!AA11/Supuestos!$D$10</f>
+        <v>43666.6666666667</v>
+      </c>
+      <c r="S11" s="60" t="n">
+        <f aca="false">SUM(G11:R11)</f>
+        <v>488000</v>
+      </c>
+      <c r="T11" s="37" t="str">
+        <f aca="false">IF(E11="Expatriado","Empresa cubre / neutraliza impuesto del país de trabajo",IF(E11="Repatriado","Empleado asume impuesto personal","Definir paquete"))</f>
+        <v>Empresa cubre / neutraliza impuesto del país de trabajo</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C12" s="29" t="str">
+        <f aca="false">Personal!E12</f>
+        <v>Juan Conde</v>
+      </c>
+      <c r="D12" s="29" t="str">
+        <f aca="false">Personal!D12</f>
+        <v>EPCM &amp; Engineering Manager</v>
+      </c>
+      <c r="E12" s="29" t="str">
+        <f aca="false">Personal!V12</f>
+        <v>Expatriado</v>
+      </c>
+      <c r="F12" s="29" t="str">
+        <f aca="false">Personal!W12</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <f aca="false">Personal!U12/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="H12" s="20" t="n">
+        <f aca="false">Personal!U12/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="I12" s="20" t="n">
+        <f aca="false">Personal!U12/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="J12" s="20" t="n">
+        <f aca="false">Personal!U12/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="K12" s="20" t="n">
+        <f aca="false">Personal!U12/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="L12" s="20" t="n">
+        <f aca="false">Personal!U12/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="M12" s="20" t="n">
+        <f aca="false">Personal!AA12/Supuestos!$D$10+Personal!Z12</f>
+        <v>27100</v>
+      </c>
+      <c r="N12" s="20" t="n">
+        <f aca="false">Personal!AA12/Supuestos!$D$10</f>
+        <v>27100</v>
+      </c>
+      <c r="O12" s="20" t="n">
+        <f aca="false">Personal!AA12/Supuestos!$D$10</f>
+        <v>27100</v>
+      </c>
+      <c r="P12" s="20" t="n">
+        <f aca="false">Personal!AA12/Supuestos!$D$10</f>
+        <v>27100</v>
+      </c>
+      <c r="Q12" s="20" t="n">
+        <f aca="false">Personal!AA12/Supuestos!$D$10</f>
+        <v>27100</v>
+      </c>
+      <c r="R12" s="20" t="n">
+        <f aca="false">Personal!AA12/Supuestos!$D$10</f>
+        <v>27100</v>
+      </c>
+      <c r="S12" s="61" t="n">
+        <f aca="false">SUM(G12:R12)</f>
+        <v>303600</v>
+      </c>
+      <c r="T12" s="39" t="str">
+        <f aca="false">IF(E12="Expatriado","Empresa cubre / neutraliza impuesto del país de trabajo",IF(E12="Repatriado","Empleado asume impuesto personal","Definir paquete"))</f>
+        <v>Empresa cubre / neutraliza impuesto del país de trabajo</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C13" s="29" t="str">
+        <f aca="false">Personal!E13</f>
+        <v>Alexander Stulme</v>
+      </c>
+      <c r="D13" s="29" t="str">
+        <f aca="false">Personal!D13</f>
+        <v>Drilling &amp; Well Services Manager</v>
+      </c>
+      <c r="E13" s="29" t="str">
+        <f aca="false">Personal!V13</f>
+        <v>Expatriado</v>
+      </c>
+      <c r="F13" s="29" t="str">
+        <f aca="false">Personal!W13</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G13" s="10" t="n">
+        <f aca="false">Personal!U13/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="H13" s="20" t="n">
+        <f aca="false">Personal!U13/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="I13" s="20" t="n">
+        <f aca="false">Personal!U13/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="J13" s="20" t="n">
+        <f aca="false">Personal!U13/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="K13" s="20" t="n">
+        <f aca="false">Personal!U13/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="L13" s="20" t="n">
+        <f aca="false">Personal!U13/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="M13" s="20" t="n">
+        <f aca="false">Personal!AA13/Supuestos!$D$10+Personal!Z13</f>
+        <v>23500</v>
+      </c>
+      <c r="N13" s="20" t="n">
+        <f aca="false">Personal!AA13/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="O13" s="20" t="n">
+        <f aca="false">Personal!AA13/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="P13" s="20" t="n">
+        <f aca="false">Personal!AA13/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="Q13" s="20" t="n">
+        <f aca="false">Personal!AA13/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="R13" s="20" t="n">
+        <f aca="false">Personal!AA13/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="S13" s="61" t="n">
+        <f aca="false">SUM(G13:R13)</f>
+        <v>264000</v>
+      </c>
+      <c r="T13" s="39" t="str">
+        <f aca="false">IF(E13="Expatriado","Empresa cubre / neutraliza impuesto del país de trabajo",IF(E13="Repatriado","Empleado asume impuesto personal","Definir paquete"))</f>
+        <v>Empresa cubre / neutraliza impuesto del país de trabajo</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C14" s="29" t="str">
+        <f aca="false">Personal!E14</f>
+        <v>Félix Valderrama</v>
+      </c>
+      <c r="D14" s="29" t="str">
+        <f aca="false">Personal!D14</f>
+        <v>Operations &amp; Maintenance Manager</v>
+      </c>
+      <c r="E14" s="29" t="str">
+        <f aca="false">Personal!V14</f>
+        <v>Expatriado</v>
+      </c>
+      <c r="F14" s="29" t="str">
+        <f aca="false">Personal!W14</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <f aca="false">Personal!U14/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="H14" s="20" t="n">
+        <f aca="false">Personal!U14/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="I14" s="20" t="n">
+        <f aca="false">Personal!U14/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="J14" s="20" t="n">
+        <f aca="false">Personal!U14/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="K14" s="20" t="n">
+        <f aca="false">Personal!U14/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="L14" s="20" t="n">
+        <f aca="false">Personal!U14/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="M14" s="20" t="n">
+        <f aca="false">Personal!AA14/Supuestos!$D$10+Personal!Z14</f>
+        <v>27100</v>
+      </c>
+      <c r="N14" s="20" t="n">
+        <f aca="false">Personal!AA14/Supuestos!$D$10</f>
+        <v>27100</v>
+      </c>
+      <c r="O14" s="20" t="n">
+        <f aca="false">Personal!AA14/Supuestos!$D$10</f>
+        <v>27100</v>
+      </c>
+      <c r="P14" s="20" t="n">
+        <f aca="false">Personal!AA14/Supuestos!$D$10</f>
+        <v>27100</v>
+      </c>
+      <c r="Q14" s="20" t="n">
+        <f aca="false">Personal!AA14/Supuestos!$D$10</f>
+        <v>27100</v>
+      </c>
+      <c r="R14" s="20" t="n">
+        <f aca="false">Personal!AA14/Supuestos!$D$10</f>
+        <v>27100</v>
+      </c>
+      <c r="S14" s="61" t="n">
+        <f aca="false">SUM(G14:R14)</f>
+        <v>303600</v>
+      </c>
+      <c r="T14" s="39" t="str">
+        <f aca="false">IF(E14="Expatriado","Empresa cubre / neutraliza impuesto del país de trabajo",IF(E14="Repatriado","Empleado asume impuesto personal","Definir paquete"))</f>
+        <v>Empresa cubre / neutraliza impuesto del país de trabajo</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C15" s="29" t="str">
+        <f aca="false">Personal!E15</f>
+        <v>Alan McKeon</v>
+      </c>
+      <c r="D15" s="29" t="str">
+        <f aca="false">Personal!D15</f>
+        <v>Technical Manager (Geosciences)</v>
+      </c>
+      <c r="E15" s="29" t="str">
+        <f aca="false">Personal!V15</f>
+        <v>Expatriado</v>
+      </c>
+      <c r="F15" s="29" t="str">
+        <f aca="false">Personal!W15</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <f aca="false">Personal!U15/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <f aca="false">Personal!U15/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="I15" s="20" t="n">
+        <f aca="false">Personal!U15/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="J15" s="20" t="n">
+        <f aca="false">Personal!U15/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="K15" s="20" t="n">
+        <f aca="false">Personal!U15/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="L15" s="20" t="n">
+        <f aca="false">Personal!U15/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="M15" s="20" t="n">
+        <f aca="false">Personal!AA15/Supuestos!$D$10+Personal!Z15</f>
+        <v>23500</v>
+      </c>
+      <c r="N15" s="20" t="n">
+        <f aca="false">Personal!AA15/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="O15" s="20" t="n">
+        <f aca="false">Personal!AA15/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="P15" s="20" t="n">
+        <f aca="false">Personal!AA15/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="Q15" s="20" t="n">
+        <f aca="false">Personal!AA15/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="R15" s="20" t="n">
+        <f aca="false">Personal!AA15/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="S15" s="61" t="n">
+        <f aca="false">SUM(G15:R15)</f>
+        <v>264000</v>
+      </c>
+      <c r="T15" s="39" t="str">
+        <f aca="false">IF(E15="Expatriado","Empresa cubre / neutraliza impuesto del país de trabajo",IF(E15="Repatriado","Empleado asume impuesto personal","Definir paquete"))</f>
+        <v>Empresa cubre / neutraliza impuesto del país de trabajo</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C16" s="29" t="str">
+        <f aca="false">Personal!E16</f>
+        <v>JJI</v>
+      </c>
+      <c r="D16" s="29" t="str">
+        <f aca="false">Personal!D16</f>
+        <v>Reservoir Engineer</v>
+      </c>
+      <c r="E16" s="29" t="str">
+        <f aca="false">Personal!V16</f>
+        <v>Expatriado</v>
+      </c>
+      <c r="F16" s="29" t="str">
+        <f aca="false">Personal!W16</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G16" s="10" t="n">
+        <f aca="false">Personal!U16/Supuestos!$D$9</f>
+        <v>14500</v>
+      </c>
+      <c r="H16" s="20" t="n">
+        <f aca="false">Personal!U16/Supuestos!$D$9</f>
+        <v>14500</v>
+      </c>
+      <c r="I16" s="20" t="n">
+        <f aca="false">Personal!U16/Supuestos!$D$9</f>
+        <v>14500</v>
+      </c>
+      <c r="J16" s="20" t="n">
+        <f aca="false">Personal!U16/Supuestos!$D$9</f>
+        <v>14500</v>
+      </c>
+      <c r="K16" s="20" t="n">
+        <f aca="false">Personal!U16/Supuestos!$D$9</f>
+        <v>14500</v>
+      </c>
+      <c r="L16" s="20" t="n">
+        <f aca="false">Personal!U16/Supuestos!$D$9</f>
+        <v>14500</v>
+      </c>
+      <c r="M16" s="20" t="n">
+        <f aca="false">Personal!AA16/Supuestos!$D$10+Personal!Z16</f>
+        <v>16166.6666666667</v>
+      </c>
+      <c r="N16" s="20" t="n">
+        <f aca="false">Personal!AA16/Supuestos!$D$10</f>
+        <v>16166.6666666667</v>
+      </c>
+      <c r="O16" s="20" t="n">
+        <f aca="false">Personal!AA16/Supuestos!$D$10</f>
+        <v>16166.6666666667</v>
+      </c>
+      <c r="P16" s="20" t="n">
+        <f aca="false">Personal!AA16/Supuestos!$D$10</f>
+        <v>16166.6666666667</v>
+      </c>
+      <c r="Q16" s="20" t="n">
+        <f aca="false">Personal!AA16/Supuestos!$D$10</f>
+        <v>16166.6666666667</v>
+      </c>
+      <c r="R16" s="20" t="n">
+        <f aca="false">Personal!AA16/Supuestos!$D$10</f>
+        <v>16166.6666666667</v>
+      </c>
+      <c r="S16" s="61" t="n">
+        <f aca="false">SUM(G16:R16)</f>
+        <v>184000</v>
+      </c>
+      <c r="T16" s="39" t="str">
+        <f aca="false">IF(E16="Expatriado","Empresa cubre / neutraliza impuesto del país de trabajo",IF(E16="Repatriado","Empleado asume impuesto personal","Definir paquete"))</f>
+        <v>Empresa cubre / neutraliza impuesto del país de trabajo</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C17" s="29" t="str">
+        <f aca="false">Personal!E17</f>
+        <v>Marcelo Dantas</v>
+      </c>
+      <c r="D17" s="29" t="str">
+        <f aca="false">Personal!D17</f>
+        <v>Rig Company Man</v>
+      </c>
+      <c r="E17" s="29" t="str">
+        <f aca="false">Personal!V17</f>
+        <v>Expatriado</v>
+      </c>
+      <c r="F17" s="29" t="str">
+        <f aca="false">Personal!W17</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G17" s="10" t="n">
+        <f aca="false">Personal!U17/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="H17" s="20" t="n">
+        <f aca="false">Personal!U17/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="I17" s="20" t="n">
+        <f aca="false">Personal!U17/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="J17" s="20" t="n">
+        <f aca="false">Personal!U17/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="K17" s="20" t="n">
+        <f aca="false">Personal!U17/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="L17" s="20" t="n">
+        <f aca="false">Personal!U17/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="M17" s="20" t="n">
+        <f aca="false">Personal!AA17/Supuestos!$D$10+Personal!Z17</f>
+        <v>23500</v>
+      </c>
+      <c r="N17" s="20" t="n">
+        <f aca="false">Personal!AA17/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="O17" s="20" t="n">
+        <f aca="false">Personal!AA17/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="P17" s="20" t="n">
+        <f aca="false">Personal!AA17/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="Q17" s="20" t="n">
+        <f aca="false">Personal!AA17/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="R17" s="20" t="n">
+        <f aca="false">Personal!AA17/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="S17" s="61" t="n">
+        <f aca="false">SUM(G17:R17)</f>
+        <v>264000</v>
+      </c>
+      <c r="T17" s="39" t="str">
+        <f aca="false">IF(E17="Expatriado","Empresa cubre / neutraliza impuesto del país de trabajo",IF(E17="Repatriado","Empleado asume impuesto personal","Definir paquete"))</f>
+        <v>Empresa cubre / neutraliza impuesto del país de trabajo</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C18" s="29" t="str">
+        <f aca="false">Personal!E18</f>
+        <v>Jose Miguel</v>
+      </c>
+      <c r="D18" s="29" t="str">
+        <f aca="false">Personal!D18</f>
+        <v>Planning &amp; PMO</v>
+      </c>
+      <c r="E18" s="29" t="str">
+        <f aca="false">Personal!V18</f>
+        <v>Expatriado</v>
+      </c>
+      <c r="F18" s="29" t="str">
+        <f aca="false">Personal!W18</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <f aca="false">Personal!U18/Supuestos!$D$9</f>
+        <v>6266.66666666667</v>
+      </c>
+      <c r="H18" s="20" t="n">
+        <f aca="false">Personal!U18/Supuestos!$D$9</f>
+        <v>6266.66666666667</v>
+      </c>
+      <c r="I18" s="20" t="n">
+        <f aca="false">Personal!U18/Supuestos!$D$9</f>
+        <v>6266.66666666667</v>
+      </c>
+      <c r="J18" s="20" t="n">
+        <f aca="false">Personal!U18/Supuestos!$D$9</f>
+        <v>6266.66666666667</v>
+      </c>
+      <c r="K18" s="20" t="n">
+        <f aca="false">Personal!U18/Supuestos!$D$9</f>
+        <v>6266.66666666667</v>
+      </c>
+      <c r="L18" s="20" t="n">
+        <f aca="false">Personal!U18/Supuestos!$D$9</f>
+        <v>6266.66666666667</v>
+      </c>
+      <c r="M18" s="20" t="n">
+        <f aca="false">Personal!AA18/Supuestos!$D$10+Personal!Z18</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="N18" s="20" t="n">
+        <f aca="false">Personal!AA18/Supuestos!$D$10</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="O18" s="20" t="n">
+        <f aca="false">Personal!AA18/Supuestos!$D$10</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="P18" s="20" t="n">
+        <f aca="false">Personal!AA18/Supuestos!$D$10</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="Q18" s="20" t="n">
+        <f aca="false">Personal!AA18/Supuestos!$D$10</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="R18" s="20" t="n">
+        <f aca="false">Personal!AA18/Supuestos!$D$10</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="S18" s="61" t="n">
+        <f aca="false">SUM(G18:R18)</f>
+        <v>81200</v>
+      </c>
+      <c r="T18" s="39" t="str">
+        <f aca="false">IF(E18="Expatriado","Empresa cubre / neutraliza impuesto del país de trabajo",IF(E18="Repatriado","Empleado asume impuesto personal","Definir paquete"))</f>
+        <v>Empresa cubre / neutraliza impuesto del país de trabajo</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C19" s="30" t="str">
+        <f aca="false">Personal!E19</f>
+        <v>Leticia Almeida</v>
+      </c>
+      <c r="D19" s="30" t="str">
+        <f aca="false">Personal!D19</f>
+        <v>Operations Support</v>
+      </c>
+      <c r="E19" s="30" t="str">
+        <f aca="false">Personal!V19</f>
+        <v>Expatriado</v>
+      </c>
+      <c r="F19" s="30" t="str">
+        <f aca="false">Personal!W19</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G19" s="23" t="n">
+        <f aca="false">Personal!U19/Supuestos!$D$9</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="H19" s="24" t="n">
+        <f aca="false">Personal!U19/Supuestos!$D$9</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="I19" s="24" t="n">
+        <f aca="false">Personal!U19/Supuestos!$D$9</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="J19" s="24" t="n">
+        <f aca="false">Personal!U19/Supuestos!$D$9</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="K19" s="24" t="n">
+        <f aca="false">Personal!U19/Supuestos!$D$9</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="L19" s="24" t="n">
+        <f aca="false">Personal!U19/Supuestos!$D$9</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="M19" s="24" t="n">
+        <f aca="false">Personal!AA19/Supuestos!$D$10+Personal!Z19</f>
+        <v>7933.33333333333</v>
+      </c>
+      <c r="N19" s="24" t="n">
+        <f aca="false">Personal!AA19/Supuestos!$D$10</f>
+        <v>7933.33333333333</v>
+      </c>
+      <c r="O19" s="24" t="n">
+        <f aca="false">Personal!AA19/Supuestos!$D$10</f>
+        <v>7933.33333333333</v>
+      </c>
+      <c r="P19" s="24" t="n">
+        <f aca="false">Personal!AA19/Supuestos!$D$10</f>
+        <v>7933.33333333333</v>
+      </c>
+      <c r="Q19" s="24" t="n">
+        <f aca="false">Personal!AA19/Supuestos!$D$10</f>
+        <v>7933.33333333333</v>
+      </c>
+      <c r="R19" s="24" t="n">
+        <f aca="false">Personal!AA19/Supuestos!$D$10</f>
+        <v>7933.33333333333</v>
+      </c>
+      <c r="S19" s="62" t="n">
+        <f aca="false">SUM(G19:R19)</f>
+        <v>91200</v>
+      </c>
+      <c r="T19" s="41" t="str">
+        <f aca="false">IF(E19="Expatriado","Empresa cubre / neutraliza impuesto del país de trabajo",IF(E19="Repatriado","Empleado asume impuesto personal","Definir paquete"))</f>
+        <v>Empresa cubre / neutraliza impuesto del país de trabajo</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C21" s="57" t="s">
+        <v>164</v>
+      </c>
+      <c r="D21" s="57"/>
+      <c r="E21" s="57"/>
+      <c r="F21" s="57"/>
+      <c r="G21" s="58" t="n">
+        <f aca="false">SUM(G11:G19)</f>
+        <v>174200</v>
+      </c>
+      <c r="H21" s="59" t="n">
+        <f aca="false">SUM(H11:H19)</f>
+        <v>174200</v>
+      </c>
+      <c r="I21" s="59" t="n">
+        <f aca="false">SUM(I11:I19)</f>
+        <v>174200</v>
+      </c>
+      <c r="J21" s="59" t="n">
+        <f aca="false">SUM(J11:J19)</f>
+        <v>174200</v>
+      </c>
+      <c r="K21" s="59" t="n">
+        <f aca="false">SUM(K11:K19)</f>
+        <v>174200</v>
+      </c>
+      <c r="L21" s="59" t="n">
+        <f aca="false">SUM(L11:L19)</f>
+        <v>174200</v>
+      </c>
+      <c r="M21" s="59" t="n">
+        <f aca="false">SUM(M11:M19)</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="N21" s="59" t="n">
+        <f aca="false">SUM(N11:N19)</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="O21" s="59" t="n">
+        <f aca="false">SUM(O11:O19)</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="P21" s="59" t="n">
+        <f aca="false">SUM(P11:P19)</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="Q21" s="59" t="n">
+        <f aca="false">SUM(Q11:Q19)</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="R21" s="59" t="n">
+        <f aca="false">SUM(R11:R19)</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="S21" s="59" t="n">
+        <f aca="false">SUM(S11:S19)</f>
+        <v>2243600</v>
+      </c>
+      <c r="T21" s="56"/>
+    </row>
+    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C24" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4"/>
+      <c r="Q24" s="4"/>
+      <c r="R24" s="4"/>
+      <c r="S24" s="4"/>
+      <c r="T24" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C25" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="K25" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="L25" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="M25" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="N25" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="O25" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="P25" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q25" s="5" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C26" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="E26" s="18" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="F26" s="18" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="G26" s="18" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="H26" s="18" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="I26" s="18" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="J26" s="60" t="n">
+        <f aca="false">M21</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="K26" s="60" t="n">
+        <f aca="false">N21</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="L26" s="60" t="n">
+        <f aca="false">O21</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="M26" s="60" t="n">
+        <f aca="false">P21</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="N26" s="60" t="n">
+        <f aca="false">Q21</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="O26" s="60" t="n">
+        <f aca="false">R21</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="P26" s="60" t="n">
+        <f aca="false">SUM(D26:O26)</f>
+        <v>2243600</v>
+      </c>
+      <c r="Q26" s="8" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C27" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="D27" s="10" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="E27" s="20" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="F27" s="20" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="G27" s="20" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="H27" s="20" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="I27" s="20" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="J27" s="20" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!I11:I19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$13)/12</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="K27" s="20" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!I11:I19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$13)/12</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="L27" s="20" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!I11:I19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$13)/12</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="M27" s="20" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!I11:I19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$13)/12</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="N27" s="20" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!I11:I19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$13)/12</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="O27" s="20" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!I11:I19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$13)/12</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="P27" s="21" t="n">
+        <f aca="false">SUM(D27:O27)</f>
+        <v>2243600</v>
+      </c>
+      <c r="Q27" s="11" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C28" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D28" s="10" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="E28" s="20" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="F28" s="20" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="G28" s="20" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="H28" s="20" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="I28" s="20" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="J28" s="20" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12</f>
+        <v>165533.333333333</v>
+      </c>
+      <c r="K28" s="20" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12</f>
+        <v>165533.333333333</v>
+      </c>
+      <c r="L28" s="20" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12</f>
+        <v>165533.333333333</v>
+      </c>
+      <c r="M28" s="20" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12</f>
+        <v>165533.333333333</v>
+      </c>
+      <c r="N28" s="20" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12</f>
+        <v>165533.333333333</v>
+      </c>
+      <c r="O28" s="20" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!G11:G19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12</f>
+        <v>165533.333333333</v>
+      </c>
+      <c r="P28" s="21" t="n">
+        <f aca="false">SUM(D28:O28)</f>
+        <v>2038400</v>
+      </c>
+      <c r="Q28" s="11" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C29" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="D29" s="23" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="E29" s="24" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="F29" s="24" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="G29" s="24" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="H29" s="24" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="I29" s="24" t="n">
+        <f aca="false">Personal!U21/Supuestos!$D$9</f>
+        <v>174200</v>
+      </c>
+      <c r="J29" s="24" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12</f>
+        <v>149033.333333333</v>
+      </c>
+      <c r="K29" s="24" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12</f>
+        <v>149033.333333333</v>
+      </c>
+      <c r="L29" s="24" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12</f>
+        <v>149033.333333333</v>
+      </c>
+      <c r="M29" s="24" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12</f>
+        <v>149033.333333333</v>
+      </c>
+      <c r="N29" s="24" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12</f>
+        <v>149033.333333333</v>
+      </c>
+      <c r="O29" s="24" t="n">
+        <f aca="false">(SUM(Personal!F11:F19)+SUM(Personal!H11:H19)+SUM(Personal!J11:J19)+SUM(Personal!K11:K19)*Supuestos!$D$12)/12</f>
+        <v>149033.333333333</v>
+      </c>
+      <c r="P29" s="25" t="n">
+        <f aca="false">SUM(D29:O29)</f>
+        <v>1939400</v>
+      </c>
+      <c r="Q29" s="16" t="s">
+        <v>188</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="C3:T3"/>
+    <mergeCell ref="C8:T8"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="C24:T24"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 &amp;K666666Mensual | Página &amp;P de &amp;N</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="C3:K34"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -8631,7 +10011,7 @@
   <sheetData>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="1" t="s">
-        <v>159</v>
+        <v>190</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -8644,17 +10024,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="2" t="s">
-        <v>160</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C6" s="3" t="s">
-        <v>161</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C8" s="4" t="s">
-        <v>162</v>
+        <v>193</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -8667,7 +10047,7 @@
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C9" s="31" t="s">
-        <v>163</v>
+        <v>194</v>
       </c>
       <c r="D9" s="31"/>
       <c r="E9" s="31"/>
@@ -8680,7 +10060,7 @@
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C10" s="31" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="D10" s="31"/>
       <c r="E10" s="31"/>
@@ -8693,7 +10073,7 @@
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C11" s="31" t="s">
-        <v>165</v>
+        <v>196</v>
       </c>
       <c r="D11" s="31"/>
       <c r="E11" s="31"/>
@@ -8706,7 +10086,7 @@
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C12" s="31" t="s">
-        <v>166</v>
+        <v>197</v>
       </c>
       <c r="D12" s="31"/>
       <c r="E12" s="31"/>
@@ -8719,7 +10099,7 @@
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C14" s="4" t="s">
-        <v>167</v>
+        <v>198</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
@@ -8732,7 +10112,7 @@
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C15" s="31" t="s">
-        <v>168</v>
+        <v>199</v>
       </c>
       <c r="D15" s="31"/>
       <c r="E15" s="31"/>
@@ -8745,7 +10125,7 @@
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C16" s="31" t="s">
-        <v>169</v>
+        <v>200</v>
       </c>
       <c r="D16" s="31"/>
       <c r="E16" s="31"/>
@@ -8758,7 +10138,7 @@
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C17" s="31" t="s">
-        <v>170</v>
+        <v>201</v>
       </c>
       <c r="D17" s="31"/>
       <c r="E17" s="31"/>
@@ -8769,9 +10149,9 @@
       <c r="J17" s="31"/>
       <c r="K17" s="31"/>
     </row>
-    <row r="18" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C18" s="31" t="s">
-        <v>171</v>
+        <v>202</v>
       </c>
       <c r="D18" s="31"/>
       <c r="E18" s="31"/>
@@ -8782,9 +10162,9 @@
       <c r="J18" s="31"/>
       <c r="K18" s="31"/>
     </row>
-    <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C19" s="31" t="s">
-        <v>172</v>
+        <v>203</v>
       </c>
       <c r="D19" s="31"/>
       <c r="E19" s="31"/>
@@ -8795,9 +10175,22 @@
       <c r="J19" s="31"/>
       <c r="K19" s="31"/>
     </row>
+    <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C20" s="31" t="s">
+        <v>204</v>
+      </c>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="31"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="31"/>
+      <c r="I20" s="31"/>
+      <c r="J20" s="31"/>
+      <c r="K20" s="31"/>
+    </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C21" s="4" t="s">
-        <v>173</v>
+        <v>205</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
@@ -8810,7 +10203,7 @@
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C22" s="31" t="s">
-        <v>174</v>
+        <v>206</v>
       </c>
       <c r="D22" s="31"/>
       <c r="E22" s="31"/>
@@ -8823,7 +10216,7 @@
     </row>
     <row r="23" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C23" s="31" t="s">
-        <v>175</v>
+        <v>207</v>
       </c>
       <c r="D23" s="31"/>
       <c r="E23" s="31"/>
@@ -8834,9 +10227,9 @@
       <c r="J23" s="31"/>
       <c r="K23" s="31"/>
     </row>
-    <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C24" s="31" t="s">
-        <v>176</v>
+        <v>208</v>
       </c>
       <c r="D24" s="31"/>
       <c r="E24" s="31"/>
@@ -8847,9 +10240,22 @@
       <c r="J24" s="31"/>
       <c r="K24" s="31"/>
     </row>
+    <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C25" s="31" t="s">
+        <v>209</v>
+      </c>
+      <c r="D25" s="31"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="31"/>
+      <c r="G25" s="31"/>
+      <c r="H25" s="31"/>
+      <c r="I25" s="31"/>
+      <c r="J25" s="31"/>
+      <c r="K25" s="31"/>
+    </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C26" s="4" t="s">
-        <v>177</v>
+        <v>210</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4"/>
@@ -8862,7 +10268,7 @@
     </row>
     <row r="27" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C27" s="31" t="s">
-        <v>178</v>
+        <v>211</v>
       </c>
       <c r="D27" s="31"/>
       <c r="E27" s="31"/>
@@ -8875,7 +10281,7 @@
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C28" s="31" t="s">
-        <v>179</v>
+        <v>212</v>
       </c>
       <c r="D28" s="31"/>
       <c r="E28" s="31"/>
@@ -8888,7 +10294,7 @@
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C30" s="4" t="s">
-        <v>180</v>
+        <v>213</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
@@ -8900,53 +10306,53 @@
       <c r="K30" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C31" s="42" t="s">
-        <v>181</v>
-      </c>
-      <c r="D31" s="42"/>
-      <c r="E31" s="42"/>
-      <c r="F31" s="42"/>
-      <c r="G31" s="42"/>
-      <c r="H31" s="42"/>
-      <c r="I31" s="42"/>
-      <c r="J31" s="42"/>
-      <c r="K31" s="42"/>
+      <c r="C31" s="43" t="s">
+        <v>214</v>
+      </c>
+      <c r="D31" s="43"/>
+      <c r="E31" s="43"/>
+      <c r="F31" s="43"/>
+      <c r="G31" s="43"/>
+      <c r="H31" s="43"/>
+      <c r="I31" s="43"/>
+      <c r="J31" s="43"/>
+      <c r="K31" s="43"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="42"/>
-      <c r="D32" s="42"/>
-      <c r="E32" s="42"/>
-      <c r="F32" s="42"/>
-      <c r="G32" s="42"/>
-      <c r="H32" s="42"/>
-      <c r="I32" s="42"/>
-      <c r="J32" s="42"/>
-      <c r="K32" s="42"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
+      <c r="E32" s="43"/>
+      <c r="F32" s="43"/>
+      <c r="G32" s="43"/>
+      <c r="H32" s="43"/>
+      <c r="I32" s="43"/>
+      <c r="J32" s="43"/>
+      <c r="K32" s="43"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="42"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="42"/>
-      <c r="F33" s="42"/>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
-      <c r="I33" s="42"/>
-      <c r="J33" s="42"/>
-      <c r="K33" s="42"/>
+      <c r="C33" s="43"/>
+      <c r="D33" s="43"/>
+      <c r="E33" s="43"/>
+      <c r="F33" s="43"/>
+      <c r="G33" s="43"/>
+      <c r="H33" s="43"/>
+      <c r="I33" s="43"/>
+      <c r="J33" s="43"/>
+      <c r="K33" s="43"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C34" s="42"/>
-      <c r="D34" s="42"/>
-      <c r="E34" s="42"/>
-      <c r="F34" s="42"/>
-      <c r="G34" s="42"/>
-      <c r="H34" s="42"/>
-      <c r="I34" s="42"/>
-      <c r="J34" s="42"/>
-      <c r="K34" s="42"/>
+      <c r="C34" s="43"/>
+      <c r="D34" s="43"/>
+      <c r="E34" s="43"/>
+      <c r="F34" s="43"/>
+      <c r="G34" s="43"/>
+      <c r="H34" s="43"/>
+      <c r="I34" s="43"/>
+      <c r="J34" s="43"/>
+      <c r="K34" s="43"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="23">
     <mergeCell ref="C3:K3"/>
     <mergeCell ref="C8:K8"/>
     <mergeCell ref="C9:K9"/>
@@ -8959,10 +10365,12 @@
     <mergeCell ref="C17:K17"/>
     <mergeCell ref="C18:K18"/>
     <mergeCell ref="C19:K19"/>
+    <mergeCell ref="C20:K20"/>
     <mergeCell ref="C21:K21"/>
     <mergeCell ref="C22:K22"/>
     <mergeCell ref="C23:K23"/>
     <mergeCell ref="C24:K24"/>
+    <mergeCell ref="C25:K25"/>
     <mergeCell ref="C26:K26"/>
     <mergeCell ref="C27:K27"/>
     <mergeCell ref="C28:K28"/>

</xml_diff>

<commit_message>
Show selected monthly cost in personnel tab
</commit_message>
<xml_diff>
--- a/projects/PetroUrdaneta-FDP9/compensation/modelo_paquetes_personal_2_etapas.xlsx
+++ b/projects/PetroUrdaneta-FDP9/compensation/modelo_paquetes_personal_2_etapas.xlsx
@@ -18,9 +18,9 @@
     <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">Definiciones!$B$2:$K$34</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Mensual!$B$2:$T$29</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Titles" vbProcedure="false">Mensual!$10:$10</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">Personal!$B$2:$AF$21</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">Personal!$B$2:$AI$21</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">Personal!$10:$10</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Personal!$C$10:$AF$19</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Personal!$C$10:$AI$19</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Resumen!$B$2:$R$45</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Supuestos!$B$2:$J$38</definedName>
   </definedNames>
@@ -4509,7 +4509,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="218">
   <si>
     <t xml:space="preserve">Resumen ejecutivo — Paquetes de personal</t>
   </si>
@@ -4967,6 +4967,18 @@
   <si>
     <t xml:space="preserve">Decision
 Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly Cost
+M1–M6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selected Monthly
+M7+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7 incl.
+Transition</t>
   </si>
   <si>
     <t xml:space="preserve">COO / PU General Manager</t>
@@ -5967,11 +5979,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="65066025"/>
-        <c:axId val="48480607"/>
+        <c:axId val="7040921"/>
+        <c:axId val="12967970"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="65066025"/>
+        <c:axId val="7040921"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6037,7 +6049,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48480607"/>
+        <c:crossAx val="12967970"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6045,7 +6057,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="48480607"/>
+        <c:axId val="12967970"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6121,7 +6133,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65066025"/>
+        <c:crossAx val="7040921"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7503,7 +7515,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="C3:AF21"/>
+  <dimension ref="C3:AI21"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="20"/>
@@ -7533,6 +7545,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="0" width="15"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7568,6 +7583,9 @@
       <c r="AD3" s="1"/>
       <c r="AE3" s="1"/>
       <c r="AF3" s="1"/>
+      <c r="AG3" s="1"/>
+      <c r="AH3" s="1"/>
+      <c r="AI3" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="2" t="s">
@@ -7612,6 +7630,9 @@
       <c r="AD8" s="4"/>
       <c r="AE8" s="4"/>
       <c r="AF8" s="4"/>
+      <c r="AG8" s="4"/>
+      <c r="AH8" s="4"/>
+      <c r="AI8" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C10" s="5" t="s">
@@ -7704,16 +7725,25 @@
       <c r="AF10" s="5" t="s">
         <v>143</v>
       </c>
+      <c r="AG10" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="AH10" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="AI10" s="5" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C11" s="44" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="45" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="E11" s="45" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="F11" s="46" t="n">
         <v>360000</v>
@@ -7773,13 +7803,13 @@
         <v>226000</v>
       </c>
       <c r="V11" s="53" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="W11" s="53" t="s">
         <v>76</v>
       </c>
       <c r="X11" s="53" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="Y11" s="54" t="str">
         <f aca="false">IF(X11="Automático",IF(W11="Caracas","Sí",IF(W11="Maracaibo","No",IF(W11="Otro","Sí","Por definir"))),X11)</f>
@@ -7812,16 +7842,28 @@
         <f aca="false">IF(V11="Por definir","Definir paquete",IF(W11="Por definir","Definir ciudad",IF(AND(V11="Repatriado",Y11="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
+      <c r="AG11" s="50" t="n">
+        <f aca="false">U11/Supuestos!$D$9</f>
+        <v>37666.6666666667</v>
+      </c>
+      <c r="AH11" s="51" t="n">
+        <f aca="false">AA11/Supuestos!$D$10</f>
+        <v>43666.6666666667</v>
+      </c>
+      <c r="AI11" s="49" t="n">
+        <f aca="false">AH11+Z11</f>
+        <v>43666.6666666667</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C12" s="44" t="n">
         <v>2</v>
       </c>
       <c r="D12" s="45" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="E12" s="45" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="F12" s="46" t="n">
         <v>216000</v>
@@ -7881,13 +7923,13 @@
         <v>141000</v>
       </c>
       <c r="V12" s="53" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="W12" s="53" t="s">
         <v>76</v>
       </c>
       <c r="X12" s="53" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="Y12" s="54" t="str">
         <f aca="false">IF(X12="Automático",IF(W12="Caracas","Sí",IF(W12="Maracaibo","No",IF(W12="Otro","Sí","Por definir"))),X12)</f>
@@ -7920,16 +7962,28 @@
         <f aca="false">IF(V12="Por definir","Definir paquete",IF(W12="Por definir","Definir ciudad",IF(AND(V12="Repatriado",Y12="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
+      <c r="AG12" s="50" t="n">
+        <f aca="false">U12/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="AH12" s="51" t="n">
+        <f aca="false">AA12/Supuestos!$D$10</f>
+        <v>27100</v>
+      </c>
+      <c r="AI12" s="49" t="n">
+        <f aca="false">AH12+Z12</f>
+        <v>27100</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C13" s="44" t="n">
         <v>3</v>
       </c>
       <c r="D13" s="45" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E13" s="45" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F13" s="46" t="n">
         <v>180000</v>
@@ -7989,13 +8043,13 @@
         <v>123000</v>
       </c>
       <c r="V13" s="53" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="W13" s="53" t="s">
         <v>76</v>
       </c>
       <c r="X13" s="53" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="Y13" s="54" t="str">
         <f aca="false">IF(X13="Automático",IF(W13="Caracas","Sí",IF(W13="Maracaibo","No",IF(W13="Otro","Sí","Por definir"))),X13)</f>
@@ -8028,16 +8082,28 @@
         <f aca="false">IF(V13="Por definir","Definir paquete",IF(W13="Por definir","Definir ciudad",IF(AND(V13="Repatriado",Y13="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
+      <c r="AG13" s="50" t="n">
+        <f aca="false">U13/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="AH13" s="51" t="n">
+        <f aca="false">AA13/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="AI13" s="49" t="n">
+        <f aca="false">AH13+Z13</f>
+        <v>23500</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C14" s="44" t="n">
         <v>4</v>
       </c>
       <c r="D14" s="45" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E14" s="45" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="F14" s="46" t="n">
         <v>216000</v>
@@ -8097,13 +8163,13 @@
         <v>141000</v>
       </c>
       <c r="V14" s="53" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="W14" s="53" t="s">
         <v>76</v>
       </c>
       <c r="X14" s="53" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="Y14" s="54" t="str">
         <f aca="false">IF(X14="Automático",IF(W14="Caracas","Sí",IF(W14="Maracaibo","No",IF(W14="Otro","Sí","Por definir"))),X14)</f>
@@ -8136,16 +8202,28 @@
         <f aca="false">IF(V14="Por definir","Definir paquete",IF(W14="Por definir","Definir ciudad",IF(AND(V14="Repatriado",Y14="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
+      <c r="AG14" s="50" t="n">
+        <f aca="false">U14/Supuestos!$D$9</f>
+        <v>23500</v>
+      </c>
+      <c r="AH14" s="51" t="n">
+        <f aca="false">AA14/Supuestos!$D$10</f>
+        <v>27100</v>
+      </c>
+      <c r="AI14" s="49" t="n">
+        <f aca="false">AH14+Z14</f>
+        <v>27100</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C15" s="44" t="n">
         <v>5</v>
       </c>
       <c r="D15" s="45" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="E15" s="45" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F15" s="46" t="n">
         <v>180000</v>
@@ -8205,13 +8283,13 @@
         <v>123000</v>
       </c>
       <c r="V15" s="53" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="W15" s="53" t="s">
         <v>76</v>
       </c>
       <c r="X15" s="53" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="Y15" s="54" t="str">
         <f aca="false">IF(X15="Automático",IF(W15="Caracas","Sí",IF(W15="Maracaibo","No",IF(W15="Otro","Sí","Por definir"))),X15)</f>
@@ -8244,16 +8322,28 @@
         <f aca="false">IF(V15="Por definir","Definir paquete",IF(W15="Por definir","Definir ciudad",IF(AND(V15="Repatriado",Y15="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
+      <c r="AG15" s="50" t="n">
+        <f aca="false">U15/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="AH15" s="51" t="n">
+        <f aca="false">AA15/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="AI15" s="49" t="n">
+        <f aca="false">AH15+Z15</f>
+        <v>23500</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C16" s="44" t="n">
         <v>6</v>
       </c>
       <c r="D16" s="45" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="E16" s="45" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F16" s="46" t="n">
         <v>120000</v>
@@ -8313,13 +8403,13 @@
         <v>87000</v>
       </c>
       <c r="V16" s="53" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="W16" s="53" t="s">
         <v>76</v>
       </c>
       <c r="X16" s="53" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="Y16" s="54" t="str">
         <f aca="false">IF(X16="Automático",IF(W16="Caracas","Sí",IF(W16="Maracaibo","No",IF(W16="Otro","Sí","Por definir"))),X16)</f>
@@ -8352,16 +8442,28 @@
         <f aca="false">IF(V16="Por definir","Definir paquete",IF(W16="Por definir","Definir ciudad",IF(AND(V16="Repatriado",Y16="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
+      <c r="AG16" s="50" t="n">
+        <f aca="false">U16/Supuestos!$D$9</f>
+        <v>14500</v>
+      </c>
+      <c r="AH16" s="51" t="n">
+        <f aca="false">AA16/Supuestos!$D$10</f>
+        <v>16166.6666666667</v>
+      </c>
+      <c r="AI16" s="49" t="n">
+        <f aca="false">AH16+Z16</f>
+        <v>16166.6666666667</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C17" s="44" t="n">
         <v>7</v>
       </c>
       <c r="D17" s="45" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E17" s="45" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F17" s="46" t="n">
         <v>180000</v>
@@ -8421,13 +8523,13 @@
         <v>123000</v>
       </c>
       <c r="V17" s="53" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="W17" s="53" t="s">
         <v>76</v>
       </c>
       <c r="X17" s="53" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="Y17" s="54" t="str">
         <f aca="false">IF(X17="Automático",IF(W17="Caracas","Sí",IF(W17="Maracaibo","No",IF(W17="Otro","Sí","Por definir"))),X17)</f>
@@ -8460,16 +8562,28 @@
         <f aca="false">IF(V17="Por definir","Definir paquete",IF(W17="Por definir","Definir ciudad",IF(AND(V17="Repatriado",Y17="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
+      <c r="AG17" s="50" t="n">
+        <f aca="false">U17/Supuestos!$D$9</f>
+        <v>20500</v>
+      </c>
+      <c r="AH17" s="51" t="n">
+        <f aca="false">AA17/Supuestos!$D$10</f>
+        <v>23500</v>
+      </c>
+      <c r="AI17" s="49" t="n">
+        <f aca="false">AH17+Z17</f>
+        <v>23500</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C18" s="44" t="n">
         <v>8</v>
       </c>
       <c r="D18" s="45" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E18" s="45" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="F18" s="46" t="n">
         <v>48000</v>
@@ -8529,13 +8643,13 @@
         <v>37600</v>
       </c>
       <c r="V18" s="53" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="W18" s="53" t="s">
         <v>76</v>
       </c>
       <c r="X18" s="53" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="Y18" s="54" t="str">
         <f aca="false">IF(X18="Automático",IF(W18="Caracas","Sí",IF(W18="Maracaibo","No",IF(W18="Otro","Sí","Por definir"))),X18)</f>
@@ -8568,16 +8682,28 @@
         <f aca="false">IF(V18="Por definir","Definir paquete",IF(W18="Por definir","Definir ciudad",IF(AND(V18="Repatriado",Y18="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
+      <c r="AG18" s="50" t="n">
+        <f aca="false">U18/Supuestos!$D$9</f>
+        <v>6266.66666666667</v>
+      </c>
+      <c r="AH18" s="51" t="n">
+        <f aca="false">AA18/Supuestos!$D$10</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="AI18" s="49" t="n">
+        <f aca="false">AH18+Z18</f>
+        <v>7266.66666666667</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C19" s="44" t="n">
         <v>9</v>
       </c>
       <c r="D19" s="45" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E19" s="45" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F19" s="46" t="n">
         <v>48000</v>
@@ -8637,13 +8763,13 @@
         <v>43600</v>
       </c>
       <c r="V19" s="53" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="W19" s="53" t="s">
         <v>76</v>
       </c>
       <c r="X19" s="53" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="Y19" s="54" t="str">
         <f aca="false">IF(X19="Automático",IF(W19="Caracas","Sí",IF(W19="Maracaibo","No",IF(W19="Otro","Sí","Por definir"))),X19)</f>
@@ -8676,11 +8802,23 @@
         <f aca="false">IF(V19="Por definir","Definir paquete",IF(W19="Por definir","Definir ciudad",IF(AND(V19="Repatriado",Y19="Por definir"),"Definir vivienda","Completo")))</f>
         <v>Definir ciudad</v>
       </c>
+      <c r="AG19" s="50" t="n">
+        <f aca="false">U19/Supuestos!$D$9</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="AH19" s="51" t="n">
+        <f aca="false">AA19/Supuestos!$D$10</f>
+        <v>7933.33333333333</v>
+      </c>
+      <c r="AI19" s="49" t="n">
+        <f aca="false">AH19+Z19</f>
+        <v>7933.33333333333</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C21" s="56"/>
       <c r="D21" s="57" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="E21" s="57"/>
       <c r="F21" s="58" t="n">
@@ -8776,12 +8914,24 @@
         <v>2396800</v>
       </c>
       <c r="AF21" s="56"/>
+      <c r="AG21" s="59" t="n">
+        <f aca="false">SUM(AG11:AG19)</f>
+        <v>174200</v>
+      </c>
+      <c r="AH21" s="59" t="n">
+        <f aca="false">SUM(AH11:AH19)</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="AI21" s="59" t="n">
+        <f aca="false">SUM(AI11:AI19)</f>
+        <v>199733.333333333</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="C10:AF19"/>
+  <autoFilter ref="C10:AI19"/>
   <mergeCells count="3">
-    <mergeCell ref="C3:AF3"/>
-    <mergeCell ref="C8:AF8"/>
+    <mergeCell ref="C3:AI3"/>
+    <mergeCell ref="C8:AI8"/>
     <mergeCell ref="D21:E21"/>
   </mergeCells>
   <conditionalFormatting sqref="AF11:AF19">
@@ -8835,7 +8985,7 @@
   <sheetData>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -8857,17 +9007,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C6" s="3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C8" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -8901,46 +9051,46 @@
         <v>44</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="P10" s="5" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="R10" s="5" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="S10" s="5" t="s">
         <v>47</v>
       </c>
       <c r="T10" s="5" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9611,7 +9761,7 @@
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C21" s="57" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D21" s="57"/>
       <c r="E21" s="57"/>
@@ -9672,7 +9822,7 @@
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C24" s="4" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
@@ -9697,46 +9847,46 @@
         <v>30</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="L25" s="5" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="N25" s="5" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="O25" s="5" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="P25" s="5" t="s">
         <v>47</v>
       </c>
       <c r="Q25" s="5" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9796,12 +9946,12 @@
         <v>2243600</v>
       </c>
       <c r="Q26" s="8" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C27" s="19" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D27" s="10" t="n">
         <f aca="false">Personal!U21/Supuestos!$D$9</f>
@@ -9856,12 +10006,12 @@
         <v>2243600</v>
       </c>
       <c r="Q27" s="11" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C28" s="19" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D28" s="10" t="n">
         <f aca="false">Personal!U21/Supuestos!$D$9</f>
@@ -9916,12 +10066,12 @@
         <v>2038400</v>
       </c>
       <c r="Q28" s="11" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C29" s="22" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D29" s="23" t="n">
         <f aca="false">Personal!U21/Supuestos!$D$9</f>
@@ -9976,7 +10126,7 @@
         <v>1939400</v>
       </c>
       <c r="Q29" s="16" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -10011,7 +10161,7 @@
   <sheetData>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="1" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -10024,17 +10174,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C6" s="3" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C8" s="4" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -10047,7 +10197,7 @@
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C9" s="31" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D9" s="31"/>
       <c r="E9" s="31"/>
@@ -10060,7 +10210,7 @@
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C10" s="31" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D10" s="31"/>
       <c r="E10" s="31"/>
@@ -10073,7 +10223,7 @@
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C11" s="31" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D11" s="31"/>
       <c r="E11" s="31"/>
@@ -10086,7 +10236,7 @@
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C12" s="31" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D12" s="31"/>
       <c r="E12" s="31"/>
@@ -10099,7 +10249,7 @@
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C14" s="4" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
@@ -10112,7 +10262,7 @@
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C15" s="31" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D15" s="31"/>
       <c r="E15" s="31"/>
@@ -10125,7 +10275,7 @@
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C16" s="31" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D16" s="31"/>
       <c r="E16" s="31"/>
@@ -10138,7 +10288,7 @@
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C17" s="31" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D17" s="31"/>
       <c r="E17" s="31"/>
@@ -10151,7 +10301,7 @@
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C18" s="31" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D18" s="31"/>
       <c r="E18" s="31"/>
@@ -10164,7 +10314,7 @@
     </row>
     <row r="19" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C19" s="31" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D19" s="31"/>
       <c r="E19" s="31"/>
@@ -10177,7 +10327,7 @@
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C20" s="31" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D20" s="31"/>
       <c r="E20" s="31"/>
@@ -10190,7 +10340,7 @@
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C21" s="4" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
@@ -10203,7 +10353,7 @@
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C22" s="31" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D22" s="31"/>
       <c r="E22" s="31"/>
@@ -10216,7 +10366,7 @@
     </row>
     <row r="23" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C23" s="31" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D23" s="31"/>
       <c r="E23" s="31"/>
@@ -10229,7 +10379,7 @@
     </row>
     <row r="24" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C24" s="31" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D24" s="31"/>
       <c r="E24" s="31"/>
@@ -10242,7 +10392,7 @@
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C25" s="31" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D25" s="31"/>
       <c r="E25" s="31"/>
@@ -10255,7 +10405,7 @@
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C26" s="4" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4"/>
@@ -10268,7 +10418,7 @@
     </row>
     <row r="27" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C27" s="31" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D27" s="31"/>
       <c r="E27" s="31"/>
@@ -10281,7 +10431,7 @@
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C28" s="31" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D28" s="31"/>
       <c r="E28" s="31"/>
@@ -10294,7 +10444,7 @@
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C30" s="4" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
@@ -10307,7 +10457,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C31" s="43" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D31" s="43"/>
       <c r="E31" s="43"/>

</xml_diff>